<commit_message>
Record owner decisions D1-D9: AI scope OpenRouter + OpenAI only, launch fixed 1 Nov
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UjdYT5q1Qx9CXiRm3KiKua
</commit_message>
<xml_diff>
--- a/docs/sprint/YOW-November-Launch-Sprint.xlsx
+++ b/docs/sprint/YOW-November-Launch-Sprint.xlsx
@@ -1650,7 +1650,7 @@
     <row r="54">
       <c r="A54" s="242" t="inlineStr">
         <is>
-          <t>Updated 30 September: work starts 1 October. Use 'Do Now' first, then 'Plan from 1 Oct' as your daily sheet. Daily Guide rows after 6 Oct are marked Moved. Overflow checks are scheduled inside your daily caps; decisions have recommended defaults.</t>
+          <t>Updated 30 September: work starts 1 October. Use 'Do Now' first, then 'Plan from 1 Oct' as your daily sheet. Daily Guide rows after 6 Oct are marked Moved. Overflow checks are scheduled inside your daily caps; decisions D1-D8 accepted 30 Sep (AI providers: OpenRouter and OpenAI only).</t>
         </is>
       </c>
     </row>
@@ -1742,22 +1742,22 @@
       </c>
       <c r="B5" s="245" t="inlineStr">
         <is>
-          <t>Decisions (5 min)</t>
+          <t>Decisions (DONE 30 Sep)</t>
         </is>
       </c>
       <c r="C5" s="245" t="inlineStr">
         <is>
-          <t>Open the 'Decisions' sheet. Read D1-D8. Reply 'accept defaults' or tell me which to change. Nothing is blocked until 3 Oct, but earlier answers let the AI plan around them.</t>
+          <t>All defaults accepted; AI providers limited to OpenRouter and OpenAI (D5). D6: please name a fallback launch date by 25 Oct if you want one; launch stays 1 Nov. D9 (new): other providers stay in the app but are labelled 'not tested'; say if you would rather hide them.</t>
         </is>
       </c>
       <c r="D5" s="245" t="inlineStr">
         <is>
-          <t>Reply in chat</t>
+          <t>Nothing to do</t>
         </is>
       </c>
       <c r="E5" s="245" t="inlineStr">
         <is>
-          <t>Decision list</t>
+          <t>Decisions</t>
         </is>
       </c>
     </row>
@@ -3153,18 +3153,19 @@
       </c>
       <c r="D23" s="245" t="inlineStr">
         <is>
-          <t>Test every advertised AI provider with the owner's own keys: context grounding, errors/retry, secret isolation.</t>
+          <t>Test the two advertised AI providers, OpenRouter and OpenAI, with the owner's own keys: context grounding, errors/retry, secret isolation. Label all other providers 'not tested' in the app.</t>
         </is>
       </c>
       <c r="E23" s="245" t="inlineStr">
         <is>
-          <t>1. AI key isolation and cross-device sync with two real accounts; proxy transport
-2. AI chat context controls and budget awareness with real providers; grounding QA; full AI chat panel Word export</t>
+          <t>1. AI key isolation and cross-device sync with two real accounts using OpenRouter and OpenAI keys; proxy transport
+2. AI chat context controls and budget awareness with real OpenRouter and OpenAI models; grounding QA
+3. Named-provider allow-list and untested-provider labelling behave as decided in D5/D9 (no custom endpoints, no advertising of other providers)</t>
         </is>
       </c>
       <c r="F23" s="245" t="inlineStr">
         <is>
-          <t>Supply provider access without sharing secrets and run the guided provider checks (includes O07 and the D&amp;D/TTRPG AI framing checks).</t>
+          <t>Supply OpenRouter and OpenAI access without sharing secrets and run the guided provider checks (includes O07 and the D&amp;D/TTRPG AI framing checks).</t>
         </is>
       </c>
       <c r="G23" s="245" t="inlineStr">
@@ -3218,8 +3219,9 @@
       </c>
       <c r="E24" s="245" t="inlineStr">
         <is>
-          <t>1. AI provider compliance document matches the named-provider list actually tested
-2. Close the Project-type gate and Product acceptance evidence for all six types</t>
+          <t>1. Full AI chat panel saved as a project entry and exported to Word; AI Import for all six project types using OpenRouter/OpenAI
+2. docs/AI_PROVIDER_COMPLIANCE.md lists exactly OpenRouter and OpenAI as supported
+3. Close the Project-type gate and Product acceptance evidence for all six types</t>
         </is>
       </c>
       <c r="F24" s="245" t="inlineStr">
@@ -3278,10 +3280,11 @@
       </c>
       <c r="E25" s="245" t="inlineStr">
         <is>
-          <t>1. Resolve every item in marketing-copy-review/COPY_CONFLICTS.md and verify Homepage, Pricing, Features, FAQ, Download, Founders, SEO pages, emails, legal modal, llms.txt, schema and Checkout say the same facts
-2. Remove player/public-discovery implications from D&amp;D/TTRPG copy (shared projects, player portals, VTT and mobile apps are excluded)
-3. SEO deployment and Search Console sitemap validation; landing page defects
-4. Legal and promise gate: Terms/Privacy final owner review, Beta 30-day notice wording, Local Mode/expiry/quota promises</t>
+          <t>1. AI provider scope (D5/D9): every mention outside OpenRouter and OpenAI is removed from Pricing, FAQ, Features, AI overview page, llms.txt, onboarding, emails and docs/AI_PROVIDER_COMPLIANCE.md; the in-app provider picker labels the others 'not tested / not officially supported'
+2. Resolve every item in marketing-copy-review/COPY_CONFLICTS.md and verify Homepage, Pricing, Features, FAQ, Download, Founders, SEO pages, emails, legal modal, llms.txt, schema and Checkout say the same facts
+3. Remove player/public-discovery implications from D&amp;D/TTRPG copy (shared projects, player portals, VTT and mobile apps are excluded)
+4. SEO deployment and Search Console sitemap validation; landing page defects
+5. Legal and promise gate: Terms/Privacy final owner review, Beta 30-day notice wording, Local Mode/expiry/quota promises</t>
         </is>
       </c>
       <c r="F25" s="245" t="inlineStr">
@@ -8228,7 +8231,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D95"/>
+  <dimension ref="A1:D98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -9712,7 +9715,7 @@
       </c>
       <c r="B74" s="245" t="inlineStr">
         <is>
-          <t>AI key isolation and cross-device sync with two real accounts; proxy transport</t>
+          <t>AI key isolation and cross-device sync with two real accounts using OpenRouter and OpenAI keys; proxy transport</t>
         </is>
       </c>
       <c r="C74" s="245" t="inlineStr">
@@ -9734,7 +9737,7 @@
       </c>
       <c r="B75" s="245" t="inlineStr">
         <is>
-          <t>AI chat context controls and budget awareness with real providers; grounding QA; full AI chat panel Word export</t>
+          <t>AI chat context controls and budget awareness with real OpenRouter and OpenAI models; grounding QA</t>
         </is>
       </c>
       <c r="C75" s="245" t="inlineStr">
@@ -9751,17 +9754,17 @@
     <row r="76">
       <c r="A76" s="245" t="inlineStr">
         <is>
-          <t>Tue 20 Oct</t>
+          <t>Mon 19 Oct</t>
         </is>
       </c>
       <c r="B76" s="245" t="inlineStr">
         <is>
-          <t>AI provider compliance document matches the named-provider list actually tested</t>
+          <t>Named-provider allow-list and untested-provider labelling behave as decided in D5/D9 (no custom endpoints, no advertising of other providers)</t>
         </is>
       </c>
       <c r="C76" s="245" t="inlineStr">
         <is>
-          <t>docs/AI_PROVIDER_COMPLIANCE.md</t>
+          <t>Owner decision 2026-09-30</t>
         </is>
       </c>
       <c r="D76" s="245" t="inlineStr">
@@ -9778,12 +9781,12 @@
       </c>
       <c r="B77" s="245" t="inlineStr">
         <is>
-          <t>Close the Project-type gate and Product acceptance evidence for all six types</t>
+          <t>Full AI chat panel saved as a project entry and exported to Word; AI Import for all six project types using OpenRouter/OpenAI</t>
         </is>
       </c>
       <c r="C77" s="245" t="inlineStr">
         <is>
-          <t>Project-type gate</t>
+          <t>Bugs: AI chat export / To Be Implemented: AI import</t>
         </is>
       </c>
       <c r="D77" s="245" t="inlineStr">
@@ -9795,17 +9798,17 @@
     <row r="78">
       <c r="A78" s="245" t="inlineStr">
         <is>
-          <t>Wed 21 Oct</t>
+          <t>Tue 20 Oct</t>
         </is>
       </c>
       <c r="B78" s="245" t="inlineStr">
         <is>
-          <t>Resolve every item in marketing-copy-review/COPY_CONFLICTS.md and verify Homepage, Pricing, Features, FAQ, Download, Founders, SEO pages, emails, legal modal, llms.txt, schema and Checkout say the same facts</t>
+          <t>docs/AI_PROVIDER_COMPLIANCE.md lists exactly OpenRouter and OpenAI as supported</t>
         </is>
       </c>
       <c r="C78" s="245" t="inlineStr">
         <is>
-          <t>QA_PLAN Priority -1 / Marketing gate</t>
+          <t>docs/AI_PROVIDER_COMPLIANCE.md</t>
         </is>
       </c>
       <c r="D78" s="245" t="inlineStr">
@@ -9817,17 +9820,17 @@
     <row r="79">
       <c r="A79" s="245" t="inlineStr">
         <is>
-          <t>Wed 21 Oct</t>
+          <t>Tue 20 Oct</t>
         </is>
       </c>
       <c r="B79" s="245" t="inlineStr">
         <is>
-          <t>Remove player/public-discovery implications from D&amp;D/TTRPG copy (shared projects, player portals, VTT and mobile apps are excluded)</t>
+          <t>Close the Project-type gate and Product acceptance evidence for all six types</t>
         </is>
       </c>
       <c r="C79" s="245" t="inlineStr">
         <is>
-          <t>QA_PLAN Priority -1: Marketing</t>
+          <t>Project-type gate</t>
         </is>
       </c>
       <c r="D79" s="245" t="inlineStr">
@@ -9844,17 +9847,17 @@
       </c>
       <c r="B80" s="245" t="inlineStr">
         <is>
-          <t>SEO deployment and Search Console sitemap validation; landing page defects</t>
+          <t>AI provider scope (D5/D9): every mention outside OpenRouter and OpenAI is removed from Pricing, FAQ, Features, AI overview page, llms.txt, onboarding, emails and docs/AI_PROVIDER_COMPLIANCE.md; the in-app provider picker labels the others 'not tested / not officially supported'</t>
         </is>
       </c>
       <c r="C80" s="245" t="inlineStr">
         <is>
-          <t>Conditional Launch Scope: SEO basics, Landing page</t>
+          <t>Launch Required / owner decision 2026-09-30</t>
         </is>
       </c>
       <c r="D80" s="245" t="inlineStr">
         <is>
-          <t>O11</t>
+          <t>AI-only</t>
         </is>
       </c>
     </row>
@@ -9866,12 +9869,12 @@
       </c>
       <c r="B81" s="245" t="inlineStr">
         <is>
-          <t>Legal and promise gate: Terms/Privacy final owner review, Beta 30-day notice wording, Local Mode/expiry/quota promises</t>
+          <t>Resolve every item in marketing-copy-review/COPY_CONFLICTS.md and verify Homepage, Pricing, Features, FAQ, Download, Founders, SEO pages, emails, legal modal, llms.txt, schema and Checkout say the same facts</t>
         </is>
       </c>
       <c r="C81" s="245" t="inlineStr">
         <is>
-          <t>Legal and promise gate</t>
+          <t>QA_PLAN Priority -1 / Marketing gate</t>
         </is>
       </c>
       <c r="D81" s="245" t="inlineStr">
@@ -9883,17 +9886,17 @@
     <row r="82">
       <c r="A82" s="245" t="inlineStr">
         <is>
-          <t>Thu 22 Oct</t>
+          <t>Wed 21 Oct</t>
         </is>
       </c>
       <c r="B82" s="245" t="inlineStr">
         <is>
-          <t>Durable Stripe event ledger: replay every supported event at least 3 times; entitlements, dates, Founder counts, emails change exactly once</t>
+          <t>Remove player/public-discovery implications from D&amp;D/TTRPG copy (shared projects, player portals, VTT and mobile apps are excluded)</t>
         </is>
       </c>
       <c r="C82" s="245" t="inlineStr">
         <is>
-          <t>QA_PLAN Priority -1: Billing</t>
+          <t>QA_PLAN Priority -1: Marketing</t>
         </is>
       </c>
       <c r="D82" s="245" t="inlineStr">
@@ -9905,39 +9908,39 @@
     <row r="83">
       <c r="A83" s="245" t="inlineStr">
         <is>
-          <t>Thu 22 Oct</t>
+          <t>Wed 21 Oct</t>
         </is>
       </c>
       <c r="B83" s="245" t="inlineStr">
         <is>
-          <t>Price/quota matrix (GBP 10 / 99 / 299 / 6) matches Stripe test Price objects and Checkout line items; repo search for stale prices</t>
+          <t>SEO deployment and Search Console sitemap validation; landing page defects</t>
         </is>
       </c>
       <c r="C83" s="245" t="inlineStr">
         <is>
-          <t>QA_PLAN Priority -1: Billing</t>
+          <t>Conditional Launch Scope: SEO basics, Landing page</t>
         </is>
       </c>
       <c r="D83" s="245" t="inlineStr">
         <is>
-          <t>AI-only</t>
+          <t>O11</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="245" t="inlineStr">
         <is>
-          <t>Thu 22 Oct</t>
+          <t>Wed 21 Oct</t>
         </is>
       </c>
       <c r="B84" s="245" t="inlineStr">
         <is>
-          <t>Remove/migrate the temporary paid-interest 'coming soon' flow and its automatic Beta entitlement; real checkout CTAs behind a launch switch</t>
+          <t>Legal and promise gate: Terms/Privacy final owner review, Beta 30-day notice wording, Local Mode/expiry/quota promises</t>
         </is>
       </c>
       <c r="C84" s="245" t="inlineStr">
         <is>
-          <t>PAYMENT_ROADMAP section 3 / QA_PLAN Priority -1</t>
+          <t>Legal and promise gate</t>
         </is>
       </c>
       <c r="D84" s="245" t="inlineStr">
@@ -9954,7 +9957,7 @@
       </c>
       <c r="B85" s="245" t="inlineStr">
         <is>
-          <t>Founder concurrency: simultaneous checkouts never exceed the approved cap</t>
+          <t>Durable Stripe event ledger: replay every supported event at least 3 times; entitlements, dates, Founder counts, emails change exactly once</t>
         </is>
       </c>
       <c r="C85" s="245" t="inlineStr">
@@ -9976,34 +9979,34 @@
       </c>
       <c r="B86" s="245" t="inlineStr">
         <is>
-          <t>Prepare the exact Vercel test-mode secrets swap and return-to-live checklist (names only, never values)</t>
+          <t>Price/quota matrix (GBP 10 / 99 / 299 / 6) matches Stripe test Price objects and Checkout line items; repo search for stale prices</t>
         </is>
       </c>
       <c r="C86" s="245" t="inlineStr">
         <is>
-          <t>PAYMENT_ROADMAP section 2</t>
+          <t>QA_PLAN Priority -1: Billing</t>
         </is>
       </c>
       <c r="D86" s="245" t="inlineStr">
         <is>
-          <t>O12</t>
+          <t>AI-only</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="245" t="inlineStr">
         <is>
-          <t>Fri 23 Oct</t>
+          <t>Thu 22 Oct</t>
         </is>
       </c>
       <c r="B87" s="245" t="inlineStr">
         <is>
-          <t>GBP 6 hosting renewal, failure/cancel checks, async payments, out-of-order webhooks</t>
+          <t>Remove/migrate the temporary paid-interest 'coming soon' flow and its automatic Beta entitlement; real checkout CTAs behind a launch switch</t>
         </is>
       </c>
       <c r="C87" s="245" t="inlineStr">
         <is>
-          <t>PAYMENT_ROADMAP section 2 steps 10-11</t>
+          <t>PAYMENT_ROADMAP section 3 / QA_PLAN Priority -1</t>
         </is>
       </c>
       <c r="D87" s="245" t="inlineStr">
@@ -10015,17 +10018,17 @@
     <row r="88">
       <c r="A88" s="245" t="inlineStr">
         <is>
-          <t>Fri 23 Oct</t>
+          <t>Thu 22 Oct</t>
         </is>
       </c>
       <c r="B88" s="245" t="inlineStr">
         <is>
-          <t>Live-account QA of the 'Downgrade to Free' fix for manually-upgraded accounts and real Stripe portal unaffected</t>
+          <t>Founder concurrency: simultaneous checkouts never exceed the approved cap</t>
         </is>
       </c>
       <c r="C88" s="245" t="inlineStr">
         <is>
-          <t>PAYMENT_ROADMAP section 2 step 12</t>
+          <t>QA_PLAN Priority -1: Billing</t>
         </is>
       </c>
       <c r="D88" s="245" t="inlineStr">
@@ -10037,17 +10040,17 @@
     <row r="89">
       <c r="A89" s="245" t="inlineStr">
         <is>
-          <t>Sat 24 Oct</t>
+          <t>Thu 22 Oct</t>
         </is>
       </c>
       <c r="B89" s="245" t="inlineStr">
         <is>
-          <t>Return-to-live prepared: swap back to live secrets/prices/webhook is a written one-step runbook; live configuration review without a purchase</t>
+          <t>Prepare the exact Vercel test-mode secrets swap and return-to-live checklist (names only, never values)</t>
         </is>
       </c>
       <c r="C89" s="245" t="inlineStr">
         <is>
-          <t>PAYMENT_ROADMAP section 2 step 13</t>
+          <t>PAYMENT_ROADMAP section 2</t>
         </is>
       </c>
       <c r="D89" s="245" t="inlineStr">
@@ -10059,130 +10062,196 @@
     <row r="90">
       <c r="A90" s="245" t="inlineStr">
         <is>
-          <t>Sat 24 Oct</t>
+          <t>Fri 23 Oct</t>
         </is>
       </c>
       <c r="B90" s="245" t="inlineStr">
         <is>
-          <t>Prepared release sets YOW_BETA_ENROLLMENT_CLOSED=true and stamps beta_notice_started_at to the launch timestamp; existing testers keep access/exports</t>
+          <t>GBP 6 hosting renewal, failure/cancel checks, async payments, out-of-order webhooks</t>
         </is>
       </c>
       <c r="C90" s="245" t="inlineStr">
         <is>
-          <t>Owner launch handoff: Beta</t>
+          <t>PAYMENT_ROADMAP section 2 steps 10-11</t>
         </is>
       </c>
       <c r="D90" s="245" t="inlineStr">
         <is>
-          <t>O13</t>
+          <t>AI-only</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="245" t="inlineStr">
         <is>
-          <t>Sat 24 Oct</t>
+          <t>Fri 23 Oct</t>
         </is>
       </c>
       <c r="B91" s="245" t="inlineStr">
         <is>
-          <t>Support inbox and email checks: support@ and founders@ receive and can reply; welcome/reset emails come from the right sender</t>
+          <t>Live-account QA of the 'Downgrade to Free' fix for manually-upgraded accounts and real Stripe portal unaffected</t>
         </is>
       </c>
       <c r="C91" s="245" t="inlineStr">
         <is>
-          <t>Owner launch handoff: Support/privacy</t>
+          <t>PAYMENT_ROADMAP section 2 step 12</t>
         </is>
       </c>
       <c r="D91" s="245" t="inlineStr">
         <is>
-          <t>O14</t>
+          <t>AI-only</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="245" t="inlineStr">
         <is>
-          <t>Fri 30 Oct</t>
+          <t>Sat 24 Oct</t>
         </is>
       </c>
       <c r="B92" s="245" t="inlineStr">
         <is>
-          <t>Final Launch Readiness Gate table update: every gate Passed with evidence or an explicit re-decision; production-deploy checks queued for 1 Nov</t>
+          <t>Return-to-live prepared: swap back to live secrets/prices/webhook is a written one-step runbook; live configuration review without a purchase</t>
         </is>
       </c>
       <c r="C92" s="245" t="inlineStr">
         <is>
-          <t>Launch Readiness Gate</t>
+          <t>PAYMENT_ROADMAP section 2 step 13</t>
         </is>
       </c>
       <c r="D92" s="245" t="inlineStr">
         <is>
-          <t>AI-only</t>
+          <t>O12</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="245" t="inlineStr">
         <is>
-          <t>Sat 31 Oct</t>
+          <t>Sat 24 Oct</t>
         </is>
       </c>
       <c r="B93" s="245" t="inlineStr">
         <is>
-          <t>Supabase and project backups taken and restore-tested; checkout-disable switch and rollback tested on the rehearsal</t>
+          <t>Prepared release sets YOW_BETA_ENROLLMENT_CLOSED=true and stamps beta_notice_started_at to the launch timestamp; existing testers keep access/exports</t>
         </is>
       </c>
       <c r="C93" s="245" t="inlineStr">
         <is>
-          <t>QA_PLAN Priority 12</t>
+          <t>Owner launch handoff: Beta</t>
         </is>
       </c>
       <c r="D93" s="245" t="inlineStr">
         <is>
-          <t>AI-only</t>
+          <t>O13</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="245" t="inlineStr">
         <is>
-          <t>Sun 1 Nov</t>
+          <t>Sat 24 Oct</t>
         </is>
       </c>
       <c r="B94" s="245" t="inlineStr">
         <is>
-          <t>Post-deploy production checks: security headers, canonical redirect, Founder slot display, checkout, entitlement, save/export</t>
+          <t>Support inbox and email checks: support@ and founders@ receive and can reply; welcome/reset emails come from the right sender</t>
         </is>
       </c>
       <c r="C94" s="245" t="inlineStr">
         <is>
-          <t>QA_PLAN Priority 11-12</t>
+          <t>Owner launch handoff: Support/privacy</t>
         </is>
       </c>
       <c r="D94" s="245" t="inlineStr">
         <is>
-          <t>O15</t>
+          <t>O14</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="245" t="inlineStr">
         <is>
+          <t>Fri 30 Oct</t>
+        </is>
+      </c>
+      <c r="B95" s="245" t="inlineStr">
+        <is>
+          <t>Final Launch Readiness Gate table update: every gate Passed with evidence or an explicit re-decision; production-deploy checks queued for 1 Nov</t>
+        </is>
+      </c>
+      <c r="C95" s="245" t="inlineStr">
+        <is>
+          <t>Launch Readiness Gate</t>
+        </is>
+      </c>
+      <c r="D95" s="245" t="inlineStr">
+        <is>
+          <t>AI-only</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="245" t="inlineStr">
+        <is>
+          <t>Sat 31 Oct</t>
+        </is>
+      </c>
+      <c r="B96" s="245" t="inlineStr">
+        <is>
+          <t>Supabase and project backups taken and restore-tested; checkout-disable switch and rollback tested on the rehearsal</t>
+        </is>
+      </c>
+      <c r="C96" s="245" t="inlineStr">
+        <is>
+          <t>QA_PLAN Priority 12</t>
+        </is>
+      </c>
+      <c r="D96" s="245" t="inlineStr">
+        <is>
+          <t>AI-only</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="245" t="inlineStr">
+        <is>
+          <t>Sun 1 Nov</t>
+        </is>
+      </c>
+      <c r="B97" s="245" t="inlineStr">
+        <is>
+          <t>Post-deploy production checks: security headers, canonical redirect, Founder slot display, checkout, entitlement, save/export</t>
+        </is>
+      </c>
+      <c r="C97" s="245" t="inlineStr">
+        <is>
+          <t>QA_PLAN Priority 11-12</t>
+        </is>
+      </c>
+      <c r="D97" s="245" t="inlineStr">
+        <is>
+          <t>O15</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="245" t="inlineStr">
+        <is>
           <t>Mon 2 Nov</t>
         </is>
       </c>
-      <c r="B95" s="245" t="inlineStr">
+      <c r="B98" s="245" t="inlineStr">
         <is>
           <t>Search Console/analytics/support monitoring active; approved marketing prepared for the owner to publish</t>
         </is>
       </c>
-      <c r="C95" s="245" t="inlineStr">
+      <c r="C98" s="245" t="inlineStr">
         <is>
           <t>Launch plan</t>
         </is>
       </c>
-      <c r="D95" s="245" t="inlineStr">
+      <c r="D98" s="245" t="inlineStr">
         <is>
           <t>AI-only</t>
         </is>
@@ -10645,7 +10714,7 @@
       </c>
       <c r="B14" s="245" t="inlineStr">
         <is>
-          <t>Your own AI provider keys (never pasted into chat): DM/GM framing, key isolation across two accounts, context controls. Runs inside the 19-20 Oct owner blocks.</t>
+          <t>Your own OpenRouter and OpenAI keys (never pasted into chat): DM/GM framing, key isolation across two accounts, context controls. Runs inside the 19-20 Oct owner blocks. Other providers are not tested.</t>
         </is>
       </c>
       <c r="C14" s="245" t="inlineStr">
@@ -10860,7 +10929,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -10913,214 +10982,276 @@
     <row r="4">
       <c r="A4" s="245" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D5</t>
         </is>
       </c>
       <c r="B4" s="245" t="inlineStr">
         <is>
-          <t>JavaScript type checking, React-compiler warnings and stricter CI gates: do they block launch?</t>
+          <t>Which AI providers does launch advertise?</t>
         </is>
       </c>
       <c r="C4" s="245" t="inlineStr">
         <is>
-          <t>Park until after launch; quality hardening, not one of the seven blocker categories.</t>
+          <t>OpenRouter and OpenAI only.</t>
         </is>
       </c>
       <c r="D4" s="246" t="n">
-        <v>46298</v>
-      </c>
-      <c r="E4" s="245" t="inlineStr"/>
+        <v>46295</v>
+      </c>
+      <c r="E4" s="245" t="inlineStr">
+        <is>
+          <t>Advertise and support only OpenRouter and OpenAI (the providers the owner can access and test). Other providers are not advertised, not live-tested, and labelled 'not tested' in the app (default treatment, see D9).</t>
+        </is>
+      </c>
       <c r="F4" s="245" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Decided</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="245" t="inlineStr">
         <is>
-          <t>D3</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="B5" s="245" t="inlineStr">
         <is>
-          <t>Desktop vault encryption at rest: encrypt, or launch unencrypted with clear disclosure?</t>
+          <t>JavaScript type checking, React-compiler warnings and stricter CI gates: do they block launch?</t>
         </is>
       </c>
       <c r="C5" s="245" t="inlineStr">
         <is>
-          <t>Launch with disclosure and record the decision; revisit later.</t>
+          <t>Park until after launch; quality hardening, not one of the seven blocker categories.</t>
         </is>
       </c>
       <c r="D5" s="246" t="n">
-        <v>46301</v>
-      </c>
-      <c r="E5" s="245" t="inlineStr"/>
+        <v>46298</v>
+      </c>
+      <c r="E5" s="245" t="inlineStr">
+        <is>
+          <t>Accepted default: parked until after launch.</t>
+        </is>
+      </c>
       <c r="F5" s="245" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Decided</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="245" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="B6" s="245" t="inlineStr">
         <is>
-          <t>A very large scene (30k+ words) with a note attached types slowly. Fixing it properly is a large change. Build it, or launch with a documented soft limit and in-app warning?</t>
+          <t>Desktop vault encryption at rest: encrypt, or launch unencrypted with clear disclosure?</t>
         </is>
       </c>
       <c r="C6" s="245" t="inlineStr">
         <is>
-          <t>Ship a documented limit and warning; keep the large fix for after launch (not a data-loss or broken-save blocker).</t>
+          <t>Launch with disclosure and record the decision; revisit later.</t>
         </is>
       </c>
       <c r="D6" s="246" t="n">
-        <v>46307</v>
-      </c>
-      <c r="E6" s="245" t="inlineStr"/>
+        <v>46301</v>
+      </c>
+      <c r="E6" s="245" t="inlineStr">
+        <is>
+          <t>Accepted default: launch with disclosure; record the decision.</t>
+        </is>
+      </c>
       <c r="F6" s="245" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Decided</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="245" t="inlineStr">
         <is>
-          <t>D4</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="B7" s="245" t="inlineStr">
         <is>
-          <t>If Windows fails its clean-machine test on 17 Oct: delay launch, or launch Mac-only with Windows following?</t>
+          <t>A very large scene (30k+ words) with a note attached types slowly. Fixing it properly is a large change. Build it, or launch with a documented soft limit and in-app warning?</t>
         </is>
       </c>
       <c r="C7" s="245" t="inlineStr">
         <is>
-          <t>Decide now; Lifetime is promised for macOS and Windows. Recommended: delay only if Windows data-loss/save/export fails; otherwise fix and retest in the buffer.</t>
+          <t>Ship a documented limit and warning; keep the large fix for after launch (not a data-loss or broken-save blocker).</t>
         </is>
       </c>
       <c r="D7" s="246" t="n">
-        <v>46311</v>
-      </c>
-      <c r="E7" s="245" t="inlineStr"/>
+        <v>46307</v>
+      </c>
+      <c r="E7" s="245" t="inlineStr">
+        <is>
+          <t>Accepted default: ship a documented limit and in-app warning for very large scenes; full fix after launch.</t>
+        </is>
+      </c>
       <c r="F7" s="245" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Decided</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="245" t="inlineStr">
         <is>
-          <t>D5</t>
+          <t>D4</t>
         </is>
       </c>
       <c r="B8" s="245" t="inlineStr">
         <is>
-          <t>Which named AI providers does launch advertise? Only those get live-tested and appear in copy.</t>
+          <t>If Windows fails its clean-machine test on 17 Oct: delay launch, or launch Mac-only with Windows following?</t>
         </is>
       </c>
       <c r="C8" s="245" t="inlineStr">
         <is>
-          <t>List them once so 19 Oct tests exactly those.</t>
+          <t>Decide now; Lifetime is promised for macOS and Windows. Recommended: delay only if Windows data-loss/save/export fails; otherwise fix and retest in the buffer.</t>
         </is>
       </c>
       <c r="D8" s="246" t="n">
         <v>46311</v>
       </c>
-      <c r="E8" s="245" t="inlineStr"/>
+      <c r="E8" s="245" t="inlineStr">
+        <is>
+          <t>Accepted default: delay only if Windows data-loss/save/export fails; otherwise fix and retest in the buffer.</t>
+        </is>
+      </c>
       <c r="F8" s="245" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Decided</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="245" t="inlineStr">
         <is>
-          <t>D8</t>
+          <t>D9</t>
         </is>
       </c>
       <c r="B9" s="245" t="inlineStr">
         <is>
-          <t>Resume Stripe work: the roadmap parked payments (18 Sep); this sprint schedules 21-24 Oct for it.</t>
+          <t>Follow-on to D5: what happens to the other providers already in the app (Google, Anthropic, Groq, Mistral, Together)?</t>
         </is>
       </c>
       <c r="C9" s="245" t="inlineStr">
         <is>
-          <t>Confirm; PAYMENT_ROADMAP.md stays the Stripe tracker while the sprint drives the schedule.</t>
+          <t>Keep working but labelled 'not tested / not officially supported'; nothing advertised. (Alternative: hide them.)</t>
         </is>
       </c>
       <c r="D9" s="246" t="n">
-        <v>46315</v>
-      </c>
-      <c r="E9" s="245" t="inlineStr"/>
+        <v>46311</v>
+      </c>
+      <c r="E9" s="245" t="inlineStr">
+        <is>
+          <t>Accepted default (follow-on to D5): keep the other providers' code working but label them 'not tested / not officially supported' in the AI settings picker and remove them from all marketing and docs. Owner can instead ask for them to be hidden.</t>
+        </is>
+      </c>
       <c r="F9" s="245" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Decided</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="245" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>D8</t>
         </is>
       </c>
       <c r="B10" s="245" t="inlineStr">
         <is>
-          <t>Remove the temporary 'Paid plans are coming soon' interest flow when checkout goes live?</t>
+          <t>Resume Stripe work: the roadmap parked payments (18 Sep); this sprint schedules 21-24 Oct for it.</t>
         </is>
       </c>
       <c r="C10" s="245" t="inlineStr">
         <is>
-          <t>Yes, remove it; it grants automatic Beta access and conflicts with real checkout.</t>
+          <t>Confirm; PAYMENT_ROADMAP.md stays the Stripe tracker while the sprint drives the schedule.</t>
         </is>
       </c>
       <c r="D10" s="246" t="n">
-        <v>46316</v>
-      </c>
-      <c r="E10" s="245" t="inlineStr"/>
+        <v>46315</v>
+      </c>
+      <c r="E10" s="245" t="inlineStr">
+        <is>
+          <t>Accepted default: Stripe work resumes 21-25 Oct; PAYMENT_ROADMAP.md stays the tracker.</t>
+        </is>
+      </c>
       <c r="F10" s="245" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Decided</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="245" t="inlineStr">
         <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="B11" s="245" t="inlineStr">
+        <is>
+          <t>Remove the temporary 'Paid plans are coming soon' interest flow when checkout goes live?</t>
+        </is>
+      </c>
+      <c r="C11" s="245" t="inlineStr">
+        <is>
+          <t>Yes, remove it; it grants automatic Beta access and conflicts with real checkout.</t>
+        </is>
+      </c>
+      <c r="D11" s="246" t="n">
+        <v>46316</v>
+      </c>
+      <c r="E11" s="245" t="inlineStr">
+        <is>
+          <t>Accepted default: remove the 'coming soon' interest flow when checkout goes live.</t>
+        </is>
+      </c>
+      <c r="F11" s="245" t="inlineStr">
+        <is>
+          <t>Decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="245" t="inlineStr">
+        <is>
           <t>D6</t>
         </is>
       </c>
-      <c r="B11" s="245" t="inlineStr">
+      <c r="B12" s="245" t="inlineStr">
         <is>
           <t>Latest date you would still accept a launch slip, and the fallback date.</t>
         </is>
       </c>
-      <c r="C11" s="245" t="inlineStr">
+      <c r="C12" s="245" t="inlineStr">
         <is>
           <t>Pick a cut-off by 25 Oct so nothing is decided under pressure. Launch stays 1-2 Nov unless a gate fails.</t>
         </is>
       </c>
-      <c r="D11" s="246" t="n">
+      <c r="D12" s="246" t="n">
         <v>46320</v>
       </c>
-      <c r="E11" s="245" t="inlineStr"/>
-      <c r="F11" s="245" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="E12" s="245" t="inlineStr">
+        <is>
+          <t>Accepted default: launch date is fixed at 1 Nov (quiet release; public 2 Nov). Owner to name a fallback date by 25 Oct.</t>
+        </is>
+      </c>
+      <c r="F12" s="245" t="inlineStr">
+        <is>
+          <t>Decided</t>
         </is>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="F4:F11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F4:F12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Open,Decided"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Record Do Now results: support reply sender mismatch (O16/D10), leaked-password protection unavailable on plan
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UjdYT5q1Qx9CXiRm3KiKua
</commit_message>
<xml_diff>
--- a/docs/sprint/YOW-November-Launch-Sprint.xlsx
+++ b/docs/sprint/YOW-November-Launch-Sprint.xlsx
@@ -1683,7 +1683,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1742,12 +1742,12 @@
       </c>
       <c r="B5" s="245" t="inlineStr">
         <is>
-          <t>Decisions (DONE 30 Sep)</t>
+          <t>Decisions - DONE 30 Sep</t>
         </is>
       </c>
       <c r="C5" s="245" t="inlineStr">
         <is>
-          <t>All defaults accepted; AI providers limited to OpenRouter and OpenAI (D5). D6: please name a fallback launch date by 25 Oct if you want one; launch stays 1 Nov. D9 (new): other providers stay in the app but are labelled 'not tested'; say if you would rather hide them.</t>
+          <t>All defaults accepted; AI providers limited to OpenRouter and OpenAI (D5).</t>
         </is>
       </c>
       <c r="D5" s="245" t="inlineStr">
@@ -1769,22 +1769,17 @@
       </c>
       <c r="B6" s="245" t="inlineStr">
         <is>
-          <t>O14 Support inbox test (15 min)</t>
+          <t>O14 Support inbox test - DONE 30 Sep</t>
         </is>
       </c>
       <c r="C6" s="245" t="inlineStr">
         <is>
-          <t>1. From your personal email send a message to support@yourownworld.co.uk with subject 'Inbox test 1 Oct' and body 'test'.
-2. Send another to founders@yourownworld.co.uk with subject 'Inbox test founders'.
-3. Open the mailbox where YOW mail arrives. Expect both within a few minutes.
-4. Reply to each from that mailbox. Expect the replies in your personal inbox.
-Report: did both arrive (minutes), and what sender name/address the reply shows.
-Do not touch: DNS, mail settings, forwarding.</t>
+          <t>Both emails arrived. The reply showed as 'Morgan Bishop, yourownworld.admin@gmail.com' rather than support@ / founders@. Follow-up is task 6.</t>
         </is>
       </c>
       <c r="D6" s="245" t="inlineStr">
         <is>
-          <t>Your mailboxes</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E6" s="245" t="inlineStr">
@@ -1801,21 +1796,17 @@
       </c>
       <c r="B7" s="245" t="inlineStr">
         <is>
-          <t>O02 Leaked-password protection (10 min)</t>
+          <t>O02 Leaked-password protection - DONE 30 Sep</t>
         </is>
       </c>
       <c r="C7" s="245" t="inlineStr">
         <is>
-          <t>1. Open supabase.com/dashboard and open the YOW production project.
-2. In the left menu choose Authentication and look for a password-security setting called 'Prevent use of leaked passwords' (it is usually under Sign In / Providers, then Email, or under Attack Protection).
-3. If there is a toggle, turn it on and save. Expect it to show as enabled after saving.
-4. If it says it needs a paid plan or you cannot find it, take a screenshot and tell me. Do not upgrade anything.
-Do not touch: users, SQL editor, any other setting.</t>
+          <t>Not offered on your current Supabase plan, so it stays as a known Advisor warning. The AI will check your minimum password rules on 9 Oct instead. Do not upgrade the plan for this.</t>
         </is>
       </c>
       <c r="D7" s="245" t="inlineStr">
         <is>
-          <t>Supabase dashboard</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E7" s="245" t="inlineStr">
@@ -1832,14 +1823,12 @@
       </c>
       <c r="B8" s="245" t="inlineStr">
         <is>
-          <t>O06 Windows machine (10 min to decide)</t>
+          <t>O06 Windows machine - IN PROGRESS</t>
         </is>
       </c>
       <c r="C8" s="245" t="inlineStr">
         <is>
-          <t>Decide where Windows testing will happen on Sat 17 Oct for about 3 hours: a real Windows 10/11 PC, or a rented cloud Windows PC. A Windows virtual machine on your Mac is a weaker test, so avoid it for the final check.
-Tell me: which option, the Windows version, and that you have admin rights and can create a fresh Windows user.
-Do not install anything yet.</t>
+          <t>You said you will test. When ready tell me: real or cloud PC, the Windows version, that you have admin rights and can create a fresh Windows user. Needed by Sat 10 Oct. Do not install anything yet.</t>
         </is>
       </c>
       <c r="D8" s="245" t="inlineStr">
@@ -1885,6 +1874,33 @@
       <c r="E9" s="245" t="inlineStr">
         <is>
           <t>O01</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="245" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B10" s="245" t="inlineStr">
+        <is>
+          <t>O16 Replies show the YOW address (20 min)</t>
+        </is>
+      </c>
+      <c r="C10" s="245" t="inlineStr">
+        <is>
+          <t>Step 1 only for now: tell me how support@yourownworld.co.uk receives mail (for example Google Workspace, your domain registrar's forwarding, or Cloudflare email routing) and which inbox the test emails arrived in. I will then give exact 'Send mail as' steps for that setup. Decision D10: fix before launch (recommended) or accept as is.</t>
+        </is>
+      </c>
+      <c r="D10" s="245" t="inlineStr">
+        <is>
+          <t>Gmail settings + domain mail setup</t>
+        </is>
+      </c>
+      <c r="E10" s="245" t="inlineStr">
+        <is>
+          <t>O16</t>
         </is>
       </c>
     </row>
@@ -2185,7 +2201,7 @@
 4. Deploy only the authoritative Vercel billing stack; retire/quarantine the drifted legacy Supabase Edge Function Stripe copies
 5. Verify .env.example + runbook can stand up a disposable environment with no browser-exposed provider keys
 6. Scene cleanup on project delete: prepare read-only Supabase check that no scene rows remain
-7. Security Advisor leftovers: leaked-password protection and duplicate owner-only scenes policies</t>
+7. Security Advisor leftovers: leaked-password protection is NOT available on the owner's current Supabase plan (owner confirmed 30 Sep) - record it as an accepted Advisor warning and instead verify the minimum password length/strength policy; clean up the duplicate owner-only scenes policies</t>
         </is>
       </c>
       <c r="F7" s="245" t="inlineStr">
@@ -2200,11 +2216,11 @@
       </c>
       <c r="H7" s="245" t="inlineStr">
         <is>
-          <t>O14, O02, O01, O03</t>
+          <t>O01, O03, O16</t>
         </is>
       </c>
       <c r="I7" s="245" t="n">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="J7" s="245" t="inlineStr">
         <is>
@@ -8725,17 +8741,17 @@
       </c>
       <c r="B29" s="245" t="inlineStr">
         <is>
-          <t>Security Advisor leftovers: leaked-password protection and duplicate owner-only scenes policies</t>
+          <t>Security Advisor leftovers: leaked-password protection is NOT available on the owner's current Supabase plan (owner confirmed 30 Sep) - record it as an accepted Advisor warning and instead verify the minimum password length/strength policy; clean up the duplicate owner-only scenes policies</t>
         </is>
       </c>
       <c r="C29" s="245" t="inlineStr">
         <is>
-          <t>Security table / 30 Sep sprint evidence</t>
+          <t>Security table / owner 2026-09-30</t>
         </is>
       </c>
       <c r="D29" s="245" t="inlineStr">
         <is>
-          <t>O02</t>
+          <t>AI-only</t>
         </is>
       </c>
     </row>
@@ -10268,7 +10284,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -10405,10 +10421,14 @@
       </c>
       <c r="H5" s="245" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="I5" s="245" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I5" s="245" t="inlineStr">
+        <is>
+          <t>Leaked-password protection not offered on current plan (owner 30 Sep). Accepted Advisor warning; AI verifies password policy on 9 Oct.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="245" t="inlineStr">
@@ -10479,39 +10499,43 @@
       </c>
       <c r="H7" s="245" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="I7" s="245" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I7" s="245" t="inlineStr">
+        <is>
+          <t>Both test emails arrived; reply sender showed 'Morgan Bishop, yourownworld.admin@gmail.com' instead of the support@/founders@ address. Follow-up O16.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="245" t="inlineStr">
         <is>
-          <t>O04</t>
+          <t>O16</t>
         </is>
       </c>
       <c r="B8" s="245" t="inlineStr">
         <is>
-          <t>Two real browser tabs on the same test account: structured-record clobber test and the same-scene race repro.</t>
+          <t>Make replies from support@ and founders@ show the YOW address instead of the personal Gmail (Gmail 'Send mail as'). Tell me how support@ receives mail first; steps depend on that.</t>
         </is>
       </c>
       <c r="C8" s="245" t="inlineStr">
         <is>
-          <t>Two tabs, test account</t>
+          <t>Gmail settings + domain mail setup</t>
         </is>
       </c>
       <c r="D8" s="245" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="E8" s="246" t="n">
-        <v>46300</v>
+        <v>46298</v>
       </c>
       <c r="F8" s="246" t="n">
-        <v>46300</v>
+        <v>46324</v>
       </c>
       <c r="G8" s="245" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H8" s="245" t="inlineStr">
@@ -10524,21 +10548,21 @@
     <row r="9">
       <c r="A9" s="245" t="inlineStr">
         <is>
-          <t>O05</t>
+          <t>O04</t>
         </is>
       </c>
       <c r="B9" s="245" t="inlineStr">
         <is>
-          <t>Live rate-limit check: send 6 feedback requests from one connection, confirm the 6th is refused and the block clears.</t>
+          <t>Two real browser tabs on the same test account: structured-record clobber test and the same-scene race repro.</t>
         </is>
       </c>
       <c r="C9" s="245" t="inlineStr">
         <is>
-          <t>Production site (guided)</t>
+          <t>Two tabs, test account</t>
         </is>
       </c>
       <c r="D9" s="245" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="E9" s="246" t="n">
         <v>46300</v>
@@ -10548,7 +10572,7 @@
       </c>
       <c r="G9" s="245" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H9" s="245" t="inlineStr">
@@ -10561,31 +10585,31 @@
     <row r="10">
       <c r="A10" s="245" t="inlineStr">
         <is>
-          <t>O06</t>
+          <t>O05</t>
         </is>
       </c>
       <c r="B10" s="245" t="inlineStr">
         <is>
-          <t>Arrange a clean Windows PC (or rented cloud Windows PC) for 17 Oct and tell me the Windows version.</t>
+          <t>Live rate-limit check: send 6 feedback requests from one connection, confirm the 6th is refused and the block clears.</t>
         </is>
       </c>
       <c r="C10" s="245" t="inlineStr">
         <is>
-          <t>Windows machine</t>
+          <t>Production site (guided)</t>
         </is>
       </c>
       <c r="D10" s="245" t="n">
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="E10" s="246" t="n">
-        <v>46305</v>
+        <v>46300</v>
       </c>
       <c r="F10" s="246" t="n">
-        <v>46305</v>
+        <v>46300</v>
       </c>
       <c r="G10" s="245" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H10" s="245" t="inlineStr">
@@ -10598,27 +10622,27 @@
     <row r="11">
       <c r="A11" s="245" t="inlineStr">
         <is>
-          <t>O08</t>
+          <t>O06</t>
         </is>
       </c>
       <c r="B11" s="245" t="inlineStr">
         <is>
-          <t>Upload larger images to a disposable project on a real account and confirm the storage figure and cap behaviour.</t>
+          <t>Arrange a clean Windows PC (or rented cloud Windows PC) for 17 Oct and tell me the Windows version.</t>
         </is>
       </c>
       <c r="C11" s="245" t="inlineStr">
         <is>
-          <t>Test account</t>
+          <t>Windows machine</t>
         </is>
       </c>
       <c r="D11" s="245" t="n">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="E11" s="246" t="n">
         <v>46305</v>
       </c>
       <c r="F11" s="246" t="n">
-        <v>46309</v>
+        <v>46305</v>
       </c>
       <c r="G11" s="245" t="inlineStr">
         <is>
@@ -10635,31 +10659,31 @@
     <row r="12">
       <c r="A12" s="245" t="inlineStr">
         <is>
-          <t>O09</t>
+          <t>O08</t>
         </is>
       </c>
       <c r="B12" s="245" t="inlineStr">
         <is>
-          <t>On a real account with a two-project series, check Characters, Locations, Lore and Timeline sync forward to the second project.</t>
+          <t>Upload larger images to a disposable project on a real account and confirm the storage figure and cap behaviour.</t>
         </is>
       </c>
       <c r="C12" s="245" t="inlineStr">
         <is>
-          <t>Test account with a series</t>
+          <t>Test account</t>
         </is>
       </c>
       <c r="D12" s="245" t="n">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="E12" s="246" t="n">
         <v>46305</v>
       </c>
       <c r="F12" s="246" t="n">
-        <v>46311</v>
+        <v>46309</v>
       </c>
       <c r="G12" s="245" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H12" s="245" t="inlineStr">
@@ -10672,27 +10696,27 @@
     <row r="13">
       <c r="A13" s="245" t="inlineStr">
         <is>
-          <t>O10</t>
+          <t>O09</t>
         </is>
       </c>
       <c r="B13" s="245" t="inlineStr">
         <is>
-          <t>Firefox and Safari passes at phone/tablet/desktop widths plus a VoiceOver and keyboard-only run. Runs inside the 18 Oct device blocks.</t>
+          <t>On a real account with a two-project series, check Characters, Locations, Lore and Timeline sync forward to the second project.</t>
         </is>
       </c>
       <c r="C13" s="245" t="inlineStr">
         <is>
-          <t>Firefox, Safari, VoiceOver</t>
+          <t>Test account with a series</t>
         </is>
       </c>
       <c r="D13" s="245" t="n">
-        <v>90</v>
+        <v>45</v>
       </c>
       <c r="E13" s="246" t="n">
-        <v>46313</v>
+        <v>46305</v>
       </c>
       <c r="F13" s="246" t="n">
-        <v>46313</v>
+        <v>46311</v>
       </c>
       <c r="G13" s="245" t="inlineStr">
         <is>
@@ -10709,31 +10733,31 @@
     <row r="14">
       <c r="A14" s="245" t="inlineStr">
         <is>
-          <t>O07</t>
+          <t>O10</t>
         </is>
       </c>
       <c r="B14" s="245" t="inlineStr">
         <is>
-          <t>Your own OpenRouter and OpenAI keys (never pasted into chat): DM/GM framing, key isolation across two accounts, context controls. Runs inside the 19-20 Oct owner blocks. Other providers are not tested.</t>
+          <t>Firefox and Safari passes at phone/tablet/desktop widths plus a VoiceOver and keyboard-only run. Runs inside the 18 Oct device blocks.</t>
         </is>
       </c>
       <c r="C14" s="245" t="inlineStr">
         <is>
-          <t>Your AI key + two test accounts</t>
+          <t>Firefox, Safari, VoiceOver</t>
         </is>
       </c>
       <c r="D14" s="245" t="n">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="E14" s="246" t="n">
-        <v>46314</v>
+        <v>46313</v>
       </c>
       <c r="F14" s="246" t="n">
-        <v>46315</v>
+        <v>46313</v>
       </c>
       <c r="G14" s="245" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H14" s="245" t="inlineStr">
@@ -10746,31 +10770,31 @@
     <row r="15">
       <c r="A15" s="245" t="inlineStr">
         <is>
-          <t>O11</t>
+          <t>O07</t>
         </is>
       </c>
       <c r="B15" s="245" t="inlineStr">
         <is>
-          <t>Search Console: confirm the sitemap is read after deploy and request indexing for the key pages.</t>
+          <t>Your own OpenRouter and OpenAI keys (never pasted into chat): DM/GM framing, key isolation across two accounts, context controls. Runs inside the 19-20 Oct owner blocks. Other providers are not tested.</t>
         </is>
       </c>
       <c r="C15" s="245" t="inlineStr">
         <is>
-          <t>Search Console</t>
+          <t>Your AI key + two test accounts</t>
         </is>
       </c>
       <c r="D15" s="245" t="n">
-        <v>10</v>
+        <v>60</v>
       </c>
       <c r="E15" s="246" t="n">
-        <v>46319</v>
+        <v>46314</v>
       </c>
       <c r="F15" s="246" t="n">
-        <v>46321</v>
+        <v>46315</v>
       </c>
       <c r="G15" s="245" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H15" s="245" t="inlineStr">
@@ -10783,31 +10807,31 @@
     <row r="16">
       <c r="A16" s="245" t="inlineStr">
         <is>
-          <t>O12</t>
+          <t>O11</t>
         </is>
       </c>
       <c r="B16" s="245" t="inlineStr">
         <is>
-          <t>Stripe and Vercel dashboards (guided, names only): confirm live keys/prices/webhook events are ready for launch, without a purchase.</t>
+          <t>Search Console: confirm the sitemap is read after deploy and request indexing for the key pages.</t>
         </is>
       </c>
       <c r="C16" s="245" t="inlineStr">
         <is>
-          <t>Stripe + Vercel dashboards</t>
+          <t>Search Console</t>
         </is>
       </c>
       <c r="D16" s="245" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="E16" s="246" t="n">
-        <v>46320</v>
+        <v>46319</v>
       </c>
       <c r="F16" s="246" t="n">
-        <v>46324</v>
+        <v>46321</v>
       </c>
       <c r="G16" s="245" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H16" s="245" t="inlineStr">
@@ -10820,21 +10844,21 @@
     <row r="17">
       <c r="A17" s="245" t="inlineStr">
         <is>
-          <t>O13</t>
+          <t>O12</t>
         </is>
       </c>
       <c r="B17" s="245" t="inlineStr">
         <is>
-          <t>Vercel: confirm the Beta-close setting exists (name only, do not enable it yet) and approve the Beta-close timestamp plan.</t>
+          <t>Stripe and Vercel dashboards (guided, names only): confirm live keys/prices/webhook events are ready for launch, without a purchase.</t>
         </is>
       </c>
       <c r="C17" s="245" t="inlineStr">
         <is>
-          <t>Vercel dashboard (guided)</t>
+          <t>Stripe + Vercel dashboards</t>
         </is>
       </c>
       <c r="D17" s="245" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="E17" s="246" t="n">
         <v>46320</v>
@@ -10857,65 +10881,102 @@
     <row r="18">
       <c r="A18" s="245" t="inlineStr">
         <is>
+          <t>O13</t>
+        </is>
+      </c>
+      <c r="B18" s="245" t="inlineStr">
+        <is>
+          <t>Vercel: confirm the Beta-close setting exists (name only, do not enable it yet) and approve the Beta-close timestamp plan.</t>
+        </is>
+      </c>
+      <c r="C18" s="245" t="inlineStr">
+        <is>
+          <t>Vercel dashboard (guided)</t>
+        </is>
+      </c>
+      <c r="D18" s="245" t="n">
+        <v>10</v>
+      </c>
+      <c r="E18" s="246" t="n">
+        <v>46320</v>
+      </c>
+      <c r="F18" s="246" t="n">
+        <v>46324</v>
+      </c>
+      <c r="G18" s="245" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H18" s="245" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="I18" s="245" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="245" t="inlineStr">
+        <is>
           <t>O15</t>
         </is>
       </c>
-      <c r="B18" s="245" t="inlineStr">
+      <c r="B19" s="245" t="inlineStr">
         <is>
           <t>After deploy on 1 Nov: open the live site DevTools and confirm headers, the www redirect, and one Founder slot display.</t>
         </is>
       </c>
-      <c r="C18" s="245" t="inlineStr">
+      <c r="C19" s="245" t="inlineStr">
         <is>
           <t>Production site (guided)</t>
         </is>
       </c>
-      <c r="D18" s="245" t="n">
+      <c r="D19" s="245" t="n">
         <v>15</v>
       </c>
-      <c r="E18" s="246" t="n">
+      <c r="E19" s="246" t="n">
         <v>46327</v>
       </c>
-      <c r="F18" s="246" t="n">
+      <c r="F19" s="246" t="n">
         <v>46327</v>
       </c>
-      <c r="G18" s="245" t="inlineStr">
+      <c r="G19" s="245" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="H18" s="245" t="inlineStr">
+      <c r="H19" s="245" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="I18" s="245" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Total minutes</t>
-        </is>
-      </c>
-      <c r="D20">
-        <f>SUM(D4:D18)</f>
-        <v/>
-      </c>
+      <c r="I19" s="245" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="C21" t="inlineStr">
         <is>
+          <t>Total minutes</t>
+        </is>
+      </c>
+      <c r="D21">
+        <f>SUM(D4:D19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="C22" t="inlineStr">
+        <is>
           <t>Remaining minutes</t>
         </is>
       </c>
-      <c r="D21">
-        <f>SUMIF(H4:H18,"&lt;&gt;Done",D4:D18)</f>
+      <c r="D22">
+        <f>SUMIF(H4:H19,"&lt;&gt;Done",D4:D19)</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="H4:H18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H4:H19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not started,In progress,Done,Blocked"</formula1>
     </dataValidation>
   </dataValidations>
@@ -10929,7 +10990,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -11162,17 +11223,17 @@
     <row r="10">
       <c r="A10" s="245" t="inlineStr">
         <is>
-          <t>D8</t>
+          <t>D10</t>
         </is>
       </c>
       <c r="B10" s="245" t="inlineStr">
         <is>
-          <t>Resume Stripe work: the roadmap parked payments (18 Sep); this sprint schedules 21-24 Oct for it.</t>
+          <t>Replies to customers currently come from yourownworld.admin@gmail.com (shown as 'Morgan Bishop'), not support@/founders@yourownworld.co.uk, which the Terms and Privacy pages publish. Fix before launch, or accept?</t>
         </is>
       </c>
       <c r="C10" s="245" t="inlineStr">
         <is>
-          <t>Confirm; PAYMENT_ROADMAP.md stays the Stripe tracker while the sprint drives the schedule.</t>
+          <t>Fix before launch (O16): it keeps the published support address consistent and avoids replies landing in spam.</t>
         </is>
       </c>
       <c r="D10" s="246" t="n">
@@ -11180,37 +11241,37 @@
       </c>
       <c r="E10" s="245" t="inlineStr">
         <is>
-          <t>Accepted default: Stripe work resumes 21-25 Oct; PAYMENT_ROADMAP.md stays the tracker.</t>
+          <t>Open - owner to decide; default is to fix via O16.</t>
         </is>
       </c>
       <c r="F10" s="245" t="inlineStr">
         <is>
-          <t>Decided</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="245" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>D8</t>
         </is>
       </c>
       <c r="B11" s="245" t="inlineStr">
         <is>
-          <t>Remove the temporary 'Paid plans are coming soon' interest flow when checkout goes live?</t>
+          <t>Resume Stripe work: the roadmap parked payments (18 Sep); this sprint schedules 21-24 Oct for it.</t>
         </is>
       </c>
       <c r="C11" s="245" t="inlineStr">
         <is>
-          <t>Yes, remove it; it grants automatic Beta access and conflicts with real checkout.</t>
+          <t>Confirm; PAYMENT_ROADMAP.md stays the Stripe tracker while the sprint drives the schedule.</t>
         </is>
       </c>
       <c r="D11" s="246" t="n">
-        <v>46316</v>
+        <v>46315</v>
       </c>
       <c r="E11" s="245" t="inlineStr">
         <is>
-          <t>Accepted default: remove the 'coming soon' interest flow when checkout goes live.</t>
+          <t>Accepted default: Stripe work resumes 21-25 Oct; PAYMENT_ROADMAP.md stays the tracker.</t>
         </is>
       </c>
       <c r="F11" s="245" t="inlineStr">
@@ -11222,28 +11283,58 @@
     <row r="12">
       <c r="A12" s="245" t="inlineStr">
         <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="B12" s="245" t="inlineStr">
+        <is>
+          <t>Remove the temporary 'Paid plans are coming soon' interest flow when checkout goes live?</t>
+        </is>
+      </c>
+      <c r="C12" s="245" t="inlineStr">
+        <is>
+          <t>Yes, remove it; it grants automatic Beta access and conflicts with real checkout.</t>
+        </is>
+      </c>
+      <c r="D12" s="246" t="n">
+        <v>46316</v>
+      </c>
+      <c r="E12" s="245" t="inlineStr">
+        <is>
+          <t>Accepted default: remove the 'coming soon' interest flow when checkout goes live.</t>
+        </is>
+      </c>
+      <c r="F12" s="245" t="inlineStr">
+        <is>
+          <t>Decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="245" t="inlineStr">
+        <is>
           <t>D6</t>
         </is>
       </c>
-      <c r="B12" s="245" t="inlineStr">
+      <c r="B13" s="245" t="inlineStr">
         <is>
           <t>Latest date you would still accept a launch slip, and the fallback date.</t>
         </is>
       </c>
-      <c r="C12" s="245" t="inlineStr">
+      <c r="C13" s="245" t="inlineStr">
         <is>
           <t>Pick a cut-off by 25 Oct so nothing is decided under pressure. Launch stays 1-2 Nov unless a gate fails.</t>
         </is>
       </c>
-      <c r="D12" s="246" t="n">
+      <c r="D13" s="246" t="n">
         <v>46320</v>
       </c>
-      <c r="E12" s="245" t="inlineStr">
+      <c r="E13" s="245" t="inlineStr">
         <is>
           <t>Accepted default: launch date is fixed at 1 Nov (quiet release; public 2 Nov). Owner to name a fallback date by 25 Oct.</t>
         </is>
       </c>
-      <c r="F12" s="245" t="inlineStr">
+      <c r="F13" s="245" t="inlineStr">
         <is>
           <t>Decided</t>
         </is>
@@ -11251,7 +11342,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="F4:F12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F4:F13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Open,Decided"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Mark O01 and O06 done, decide D10 (fix support reply address)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UjdYT5q1Qx9CXiRm3KiKua
</commit_message>
<xml_diff>
--- a/docs/sprint/YOW-November-Launch-Sprint.xlsx
+++ b/docs/sprint/YOW-November-Launch-Sprint.xlsx
@@ -1823,17 +1823,17 @@
       </c>
       <c r="B8" s="245" t="inlineStr">
         <is>
-          <t>O06 Windows machine - IN PROGRESS</t>
+          <t>O06 Windows machine - DONE 30 Sep</t>
         </is>
       </c>
       <c r="C8" s="245" t="inlineStr">
         <is>
-          <t>You said you will test. When ready tell me: real or cloud PC, the Windows version, that you have admin rights and can create a fresh Windows user. Needed by Sat 10 Oct. Do not install anything yet.</t>
+          <t>You have a real Windows PC with admin rights. Quick extra: press the Windows key + R, type winver, press Enter, and note the Windows version shown (then close the box). Tell me whenever convenient, before 17 Oct. Do not install anything yet.</t>
         </is>
       </c>
       <c r="D8" s="245" t="inlineStr">
         <is>
-          <t>A Windows PC or cloud PC</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E8" s="245" t="inlineStr">
@@ -1850,25 +1850,17 @@
       </c>
       <c r="B9" s="245" t="inlineStr">
         <is>
-          <t>O01 Fresh-account walkthrough (40 min)</t>
+          <t>O01 Fresh-account walkthrough - DONE 30 Sep (owner-attested)</t>
         </is>
       </c>
       <c r="C9" s="245" t="inlineStr">
         <is>
-          <t>Use a private/incognito window and an email alias you control (for example yourname+yowfresh1@gmail.com). Never your owner/admin account.
-1. Open www.yourownworld.co.uk and sign up with the alias and a throwaway password. Confirm the email if asked; a welcome email should arrive.
-2. Expect a first-sign-in prompt offering 'Tour with a sample' and 'Start my own project'. Choose 'Tour with a sample'.
-3. Expect exactly one project called 'Sample Project' with a manuscript, characters and other sections. Go back to the library and count sample projects. Report the number.
-4. Dismiss the welcome tour and one section tour. Sign out.
-5. In a different browser (or a fresh profile), sign in with the same alias. Expect the tours not to reappear.
-6. Open AI settings without adding a key. Expect clear setup guidance and no error.
-Report what you saw at each step; screenshot anything different.
-Do not touch: your real projects, anyone else's account, billing.</t>
+          <t>You have run this many times, so it is recorded as passed on your word. No formal evidence was saved; if a fresh-account problem ever shows up we will reopen it.</t>
         </is>
       </c>
       <c r="D9" s="245" t="inlineStr">
         <is>
-          <t>Alias email + second browser</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E9" s="245" t="inlineStr">
@@ -1890,7 +1882,7 @@
       </c>
       <c r="C10" s="245" t="inlineStr">
         <is>
-          <t>Step 1 only for now: tell me how support@yourownworld.co.uk receives mail (for example Google Workspace, your domain registrar's forwarding, or Cloudflare email routing) and which inbox the test emails arrived in. I will then give exact 'Send mail as' steps for that setup. Decision D10: fix before launch (recommended) or accept as is.</t>
+          <t>Step 1 only for now: tell me how support@yourownworld.co.uk receives mail (for example Google Workspace, your domain registrar's forwarding, or Cloudflare email routing) and which inbox the test emails arrived in. I will then give exact 'Send mail as' steps for that setup. Decision D10: decided - fix before launch.</t>
         </is>
       </c>
       <c r="D10" s="245" t="inlineStr">
@@ -2216,11 +2208,11 @@
       </c>
       <c r="H7" s="245" t="inlineStr">
         <is>
-          <t>O01, O03, O16</t>
+          <t>O03, O16</t>
         </is>
       </c>
       <c r="I7" s="245" t="n">
-        <v>95</v>
+        <v>135</v>
       </c>
       <c r="J7" s="245" t="inlineStr">
         <is>
@@ -2645,11 +2637,11 @@
       </c>
       <c r="H14" s="245" t="inlineStr">
         <is>
-          <t>O06, O08, O09</t>
+          <t>O08, O09</t>
         </is>
       </c>
       <c r="I14" s="245" t="n">
-        <v>25</v>
+        <v>85</v>
       </c>
       <c r="J14" s="245" t="inlineStr">
         <is>
@@ -10384,10 +10376,14 @@
       </c>
       <c r="H4" s="245" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="I4" s="245" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I4" s="245" t="inlineStr">
+        <is>
+          <t>Owner-attested 30 Sep: fresh-account flow already run many times; no formal step-by-step evidence saved. Accepted as passed by owner decision.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="245" t="inlineStr">
@@ -10651,10 +10647,14 @@
       </c>
       <c r="H11" s="245" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="I11" s="245" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I11" s="245" t="inlineStr">
+        <is>
+          <t>Owner has a real Windows PC with admin rights (30 Sep). Exact Windows version to be read with winver before 17 Oct.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="245" t="inlineStr">
@@ -11241,12 +11241,12 @@
       </c>
       <c r="E10" s="245" t="inlineStr">
         <is>
-          <t>Open - owner to decide; default is to fix via O16.</t>
+          <t>Fix before launch (owner confirmed 30 Sep). Done via O16 once the owner says how support@ receives mail.</t>
         </is>
       </c>
       <c r="F10" s="245" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Decided</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
O16: record Cloudflare routing and add Gmail send-as via Resend steps
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UjdYT5q1Qx9CXiRm3KiKua
</commit_message>
<xml_diff>
--- a/docs/sprint/YOW-November-Launch-Sprint.xlsx
+++ b/docs/sprint/YOW-November-Launch-Sprint.xlsx
@@ -1877,17 +1877,33 @@
       </c>
       <c r="B10" s="245" t="inlineStr">
         <is>
-          <t>O16 Replies show the YOW address (20 min)</t>
+          <t>O16 Replies show the YOW address (about 20 min)</t>
         </is>
       </c>
       <c r="C10" s="245" t="inlineStr">
         <is>
-          <t>Step 1 only for now: tell me how support@yourownworld.co.uk receives mail (for example Google Workspace, your domain registrar's forwarding, or Cloudflare email routing) and which inbox the test emails arrived in. I will then give exact 'Send mail as' steps for that setup. Decision D10: decided - fix before launch.</t>
+          <t>Background: Cloudflare forwards support@ and founders@ to yourownworld.admin@gmail.com but cannot send mail, so Gmail replies go out as the Gmail address. The fix is to let Gmail send through Resend, which YOW already uses for its emails.
+PART A - Resend (5 min)
+1. Open resend.com/dashboard and sign in to the account YOW uses.
+2. Domains: confirm yourownworld.co.uk shows Verified. If not, stop and tell me.
+3. API Keys &gt; Create API Key. Name: Gmail send-as. Permission: Sending access. Domain: yourownworld.co.uk. Create, then copy the key (shown once). NEVER paste it into this chat or any document; you will paste it only into Gmail in Part B. Do not reuse or delete YOW's existing keys.
+PART B - Gmail, signed in as yourownworld.admin@gmail.com (10 min)
+1. Gear icon &gt; See all settings &gt; Accounts and Import &gt; Send mail as &gt; Add another email address.
+2. Name: YOW Support. Email: support@yourownworld.co.uk. Keep 'Treat as an alias' ticked. Next Step.
+3. SMTP server: smtp.resend.com. Port: 465. Username: resend. Password: the key from Part A. Choose 'Secured connection using SSL'. Add Account.
+4. Gmail sends a confirmation email to support@; Cloudflare forwards it to the same inbox. Open it and click the link (or enter the code).
+5. Repeat steps 1-4 for founders@yourownworld.co.uk with Name: YOW Founders.
+6. Still on Accounts and Import, under 'When replying to a message', choose 'Reply from the same address the message was sent to'. Save.
+PART C - test (5 min)
+1. From your personal email, send a message to support@yourownworld.co.uk. Reply to it from yourownworld.admin@gmail.com.
+2. In your personal inbox, expect the sender to read 'YOW Support &lt;support@yourownworld.co.uk&gt;' and the message to land in the inbox, not spam. Repeat for founders@.
+Report: sender shown, inbox or spam, and any error text. If Gmail says authentication failed, re-check the username (resend) and the key and tell me the exact message.
+Do not touch: Cloudflare DNS or routing rules, Resend domain settings.</t>
         </is>
       </c>
       <c r="D10" s="245" t="inlineStr">
         <is>
-          <t>Gmail settings + domain mail setup</t>
+          <t>Resend dashboard + Gmail settings</t>
         </is>
       </c>
       <c r="E10" s="245" t="inlineStr">
@@ -10512,7 +10528,7 @@
       </c>
       <c r="B8" s="245" t="inlineStr">
         <is>
-          <t>Make replies from support@ and founders@ show the YOW address instead of the personal Gmail (Gmail 'Send mail as'). Tell me how support@ receives mail first; steps depend on that.</t>
+          <t>Make replies from support@ and founders@ show the YOW address: add both as Gmail 'Send mail as' aliases that send through Resend SMTP (Cloudflare Email Routing only receives). Steps are in the Do Now sheet.</t>
         </is>
       </c>
       <c r="C8" s="245" t="inlineStr">

</xml_diff>

<commit_message>
Sprint: mark 1 Oct Done in the sheet; move live Free-deletion test to 3 Oct (owner time) as overflow O17
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018H7azoA9eeUuCzXVasUVos
</commit_message>
<xml_diff>
--- a/docs/sprint/YOW-November-Launch-Sprint.xlsx
+++ b/docs/sprint/YOW-November-Launch-Sprint.xlsx
@@ -21,7 +21,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="ddd d mmm"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="13">
     <font>
@@ -2093,10 +2093,14 @@
       </c>
       <c r="K5" s="245" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="L5" s="245" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L5" s="245" t="inlineStr">
+        <is>
+          <t>Done 2026-10-01. Lifecycle built and tested: notices (Resend, ledger-first, max 20/run), grace, archive stamp (client reads cloud_archived_at), Free-account deletion (audit table, live re-check, media cleanup, max 10/run), all gated behind env settings + request flags and scheduled daily (09:15 UTC) inside the existing send-reengagement-emails function to stay within Vercel Hobby's 12 Functions. PRs 236-240; npm run qa 138 files / 1,349 tests, 0 lint errors. Migrations applied by owner. First production report: 160 accounts, 157 swept, 0 due. Notice wording owner-approved. Production edge/headers 22/22. Owner-reported live idle-logout and cross-tab auth checks passed. CARRIED to 3 Oct (O17): live end-to-end deletion test (no real email or deletion has run in production yet).</t>
+        </is>
+      </c>
       <c r="M5" s="245" t="inlineStr">
         <is>
           <t>2026-10-07</t>
@@ -2209,12 +2213,13 @@
 4. Deploy only the authoritative Vercel billing stack; retire/quarantine the drifted legacy Supabase Edge Function Stripe copies
 5. Verify .env.example + runbook can stand up a disposable environment with no browser-exposed provider keys
 6. Scene cleanup on project delete: prepare read-only Supabase check that no scene rows remain
-7. Security Advisor leftovers: leaked-password protection is NOT available on the owner's current Supabase plan (owner confirmed 30 Sep) - record it as an accepted Advisor warning and instead verify the minimum password length/strength policy; clean up the duplicate owner-only scenes policies</t>
+7. Security Advisor leftovers: leaked-password protection is NOT available on the owner's current Supabase plan (owner confirmed 30 Sep) - record it as an accepted Advisor warning and instead verify the minimum password length/strength policy; clean up the duplicate owner-only scenes policies
+8. Free-account deletion end-to-end with two designated Free test accounts (A deleted, B signs in and is not deleted): prepare the exact SQL and checklist this morning; verify all notice emails fire, the final-notice date is right, A and its stored media are deleted with an audit row, B is untouched, no real account changes (procedure in docs/QA_PLAN.md '2026-10-03 Free-account deletion end-to-end'); feeds the 4-5 Oct data-safety matrix</t>
         </is>
       </c>
       <c r="F7" s="245" t="inlineStr">
         <is>
-          <t>Provide guided production access only if needed; review the database continuity result.</t>
+          <t>Provide guided production access only if needed; review the database continuity result. Also (O17): create the two Free test accounts and run the deletion end-to-end test using the AI's SQL (about 60 min).</t>
         </is>
       </c>
       <c r="G7" s="245" t="inlineStr">
@@ -2224,11 +2229,11 @@
       </c>
       <c r="H7" s="245" t="inlineStr">
         <is>
-          <t>O03, O16</t>
+          <t>O03, O16, O17</t>
         </is>
       </c>
       <c r="I7" s="245" t="n">
-        <v>135</v>
+        <v>75</v>
       </c>
       <c r="J7" s="245" t="inlineStr">
         <is>
@@ -10968,6 +10973,43 @@
       </c>
       <c r="I19" s="245" t="inlineStr"/>
     </row>
+    <row r="20">
+      <c r="A20" s="245" t="inlineStr">
+        <is>
+          <t>O17</t>
+        </is>
+      </c>
+      <c r="B20" s="245" t="inlineStr">
+        <is>
+          <t>Create two Free test accounts (real inboxes you can read, unbilled, not Beta) and run the Free-account deletion end-to-end test: AI prepares the exact SQL and checklist (docs/QA_PLAN.md). You paste the SQL, press Run on the Vercel cron job between steps, and report what arrives in the inbox, Resend and Supabase. Pre-check that no real account is due first.</t>
+        </is>
+      </c>
+      <c r="C20" s="245" t="inlineStr">
+        <is>
+          <t>Two Free test accounts + Supabase SQL editor + Vercel cron Run button (guided)</t>
+        </is>
+      </c>
+      <c r="D20" s="245" t="n">
+        <v>60</v>
+      </c>
+      <c r="E20" s="246" t="n">
+        <v>46298</v>
+      </c>
+      <c r="F20" s="246" t="n">
+        <v>46300</v>
+      </c>
+      <c r="G20" s="245" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H20" s="245" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="I20" s="245" t="n"/>
+    </row>
     <row r="21">
       <c r="C21" t="inlineStr">
         <is>
@@ -10975,7 +11017,7 @@
         </is>
       </c>
       <c r="D21">
-        <f>SUM(D4:D19)</f>
+        <f>SUM(D4:D20)</f>
         <v/>
       </c>
     </row>
@@ -10986,7 +11028,7 @@
         </is>
       </c>
       <c r="D22">
-        <f>SUMIF(H4:H19,"&lt;&gt;Done",D4:D19)</f>
+        <f>SUMIF(H4:H20,"&lt;&gt;Done",D4:D20)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Lifecycle: fresh notice cycle for returning accounts; schedule 3 Oct deletion end-to-end test (#240)
* Lifecycle: returning accounts start a fresh notice cycle; schedule live end-to-end deletion test (4 Oct); record 1 Oct live checks

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018H7azoA9eeUuCzXVasUVos

* Sprint: mark 1 Oct Done in the sheet; move live Free-deletion test to 3 Oct (owner time) as overflow O17

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018H7azoA9eeUuCzXVasUVos

---------

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/sprint/YOW-November-Launch-Sprint.xlsx
+++ b/docs/sprint/YOW-November-Launch-Sprint.xlsx
@@ -21,7 +21,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="ddd d mmm"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="13">
     <font>
@@ -2093,10 +2093,14 @@
       </c>
       <c r="K5" s="245" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="L5" s="245" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L5" s="245" t="inlineStr">
+        <is>
+          <t>Done 2026-10-01. Lifecycle built and tested: notices (Resend, ledger-first, max 20/run), grace, archive stamp (client reads cloud_archived_at), Free-account deletion (audit table, live re-check, media cleanup, max 10/run), all gated behind env settings + request flags and scheduled daily (09:15 UTC) inside the existing send-reengagement-emails function to stay within Vercel Hobby's 12 Functions. PRs 236-240; npm run qa 138 files / 1,349 tests, 0 lint errors. Migrations applied by owner. First production report: 160 accounts, 157 swept, 0 due. Notice wording owner-approved. Production edge/headers 22/22. Owner-reported live idle-logout and cross-tab auth checks passed. CARRIED to 3 Oct (O17): live end-to-end deletion test (no real email or deletion has run in production yet).</t>
+        </is>
+      </c>
       <c r="M5" s="245" t="inlineStr">
         <is>
           <t>2026-10-07</t>
@@ -2209,12 +2213,13 @@
 4. Deploy only the authoritative Vercel billing stack; retire/quarantine the drifted legacy Supabase Edge Function Stripe copies
 5. Verify .env.example + runbook can stand up a disposable environment with no browser-exposed provider keys
 6. Scene cleanup on project delete: prepare read-only Supabase check that no scene rows remain
-7. Security Advisor leftovers: leaked-password protection is NOT available on the owner's current Supabase plan (owner confirmed 30 Sep) - record it as an accepted Advisor warning and instead verify the minimum password length/strength policy; clean up the duplicate owner-only scenes policies</t>
+7. Security Advisor leftovers: leaked-password protection is NOT available on the owner's current Supabase plan (owner confirmed 30 Sep) - record it as an accepted Advisor warning and instead verify the minimum password length/strength policy; clean up the duplicate owner-only scenes policies
+8. Free-account deletion end-to-end with two designated Free test accounts (A deleted, B signs in and is not deleted): prepare the exact SQL and checklist this morning; verify all notice emails fire, the final-notice date is right, A and its stored media are deleted with an audit row, B is untouched, no real account changes (procedure in docs/QA_PLAN.md '2026-10-03 Free-account deletion end-to-end'); feeds the 4-5 Oct data-safety matrix</t>
         </is>
       </c>
       <c r="F7" s="245" t="inlineStr">
         <is>
-          <t>Provide guided production access only if needed; review the database continuity result.</t>
+          <t>Provide guided production access only if needed; review the database continuity result. Also (O17): create the two Free test accounts and run the deletion end-to-end test using the AI's SQL (about 60 min).</t>
         </is>
       </c>
       <c r="G7" s="245" t="inlineStr">
@@ -2224,11 +2229,11 @@
       </c>
       <c r="H7" s="245" t="inlineStr">
         <is>
-          <t>O03, O16</t>
+          <t>O03, O16, O17</t>
         </is>
       </c>
       <c r="I7" s="245" t="n">
-        <v>135</v>
+        <v>75</v>
       </c>
       <c r="J7" s="245" t="inlineStr">
         <is>
@@ -10968,6 +10973,43 @@
       </c>
       <c r="I19" s="245" t="inlineStr"/>
     </row>
+    <row r="20">
+      <c r="A20" s="245" t="inlineStr">
+        <is>
+          <t>O17</t>
+        </is>
+      </c>
+      <c r="B20" s="245" t="inlineStr">
+        <is>
+          <t>Create two Free test accounts (real inboxes you can read, unbilled, not Beta) and run the Free-account deletion end-to-end test: AI prepares the exact SQL and checklist (docs/QA_PLAN.md). You paste the SQL, press Run on the Vercel cron job between steps, and report what arrives in the inbox, Resend and Supabase. Pre-check that no real account is due first.</t>
+        </is>
+      </c>
+      <c r="C20" s="245" t="inlineStr">
+        <is>
+          <t>Two Free test accounts + Supabase SQL editor + Vercel cron Run button (guided)</t>
+        </is>
+      </c>
+      <c r="D20" s="245" t="n">
+        <v>60</v>
+      </c>
+      <c r="E20" s="246" t="n">
+        <v>46298</v>
+      </c>
+      <c r="F20" s="246" t="n">
+        <v>46300</v>
+      </c>
+      <c r="G20" s="245" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H20" s="245" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="I20" s="245" t="n"/>
+    </row>
     <row r="21">
       <c r="C21" t="inlineStr">
         <is>
@@ -10975,7 +11017,7 @@
         </is>
       </c>
       <c r="D21">
-        <f>SUM(D4:D19)</f>
+        <f>SUM(D4:D20)</f>
         <v/>
       </c>
     </row>
@@ -10986,7 +11028,7 @@
         </is>
       </c>
       <c r="D22">
-        <f>SUMIF(H4:H19,"&lt;&gt;Done",D4:D19)</f>
+        <f>SUMIF(H4:H20,"&lt;&gt;Done",D4:D20)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Record the passed live Free-account deletion end-to-end test (2 Oct) in QA plan, roadmap and sprint sheet
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018H7azoA9eeUuCzXVasUVos
</commit_message>
<xml_diff>
--- a/docs/sprint/YOW-November-Launch-Sprint.xlsx
+++ b/docs/sprint/YOW-November-Launch-Sprint.xlsx
@@ -19,9 +19,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="ddd d mmm"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="13">
     <font>
@@ -2098,7 +2097,7 @@
       </c>
       <c r="L5" s="245" t="inlineStr">
         <is>
-          <t>Done 2026-10-01. Lifecycle built and tested: notices (Resend, ledger-first, max 20/run), grace, archive stamp (client reads cloud_archived_at), Free-account deletion (audit table, live re-check, media cleanup, max 10/run), all gated behind env settings + request flags and scheduled daily (09:15 UTC) inside the existing send-reengagement-emails function to stay within Vercel Hobby's 12 Functions. PRs 236-240; npm run qa 138 files / 1,349 tests, 0 lint errors. Migrations applied by owner. First production report: 160 accounts, 157 swept, 0 due. Notice wording owner-approved. Production edge/headers 22/22. Owner-reported live idle-logout and cross-tab auth checks passed. CARRIED to 3 Oct (O17): live end-to-end deletion test (no real email or deletion has run in production yet).</t>
+          <t>Done 2026-10-01. Lifecycle built and tested: notices (Resend, ledger-first, max 20/run), grace, archive stamp (client reads cloud_archived_at), Free-account deletion (audit table, live re-check, media cleanup, max 10/run), all gated behind env settings + request flags and scheduled daily (09:15 UTC) inside the existing send-reengagement-emails function to stay within Vercel Hobby's 12 Functions. PRs 236-240; npm run qa 138 files / 1,349 tests, 0 lint errors. Migrations applied by owner. First production report: 160 accounts, 157 swept, 0 due. Notice wording owner-approved. Production edge/headers 22/22. Owner-reported live idle-logout and cross-tab auth checks passed. The live end-to-end deletion test (O17) was run early and passed on 2 Oct.</t>
         </is>
       </c>
       <c r="M5" s="245" t="inlineStr">
@@ -2245,7 +2244,11 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="L7" s="245" t="inlineStr"/>
+      <c r="L7" s="245" t="inlineStr">
+        <is>
+          <t>O17 (Free-account deletion end-to-end) already done and passed on 2 Oct. See Owner Overflow O17 and docs/QA_PLAN.md. Remaining 3 Oct work is the rest of this day's assignment.</t>
+        </is>
+      </c>
       <c r="M7" s="245" t="inlineStr">
         <is>
           <t>2026-10-09</t>
@@ -11005,10 +11008,14 @@
       </c>
       <c r="H20" s="245" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="I20" s="245" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I20" s="245" t="inlineStr">
+        <is>
+          <t>Passed 2026-10-02 (run a day early). 8 notice emails arrived; cron run deleted test account A (audit row completed in 2 s, Storage folder gone); test account B signed in after the final notice and was not deleted; no real account touched. Found and fixed: Resend idempotency 409 (PR 243); emails restyled as branded HTML (PR 242). Open: view B's 4 ledger rows; check email styling in Gmail desktop/phone; delete test account B.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="C21" t="inlineStr">

</xml_diff>

<commit_message>
Record passed live Free-account deletion end-to-end test (#244)
* Record the passed live Free-account deletion end-to-end test (2 Oct) in QA plan, roadmap and sprint sheet

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018H7azoA9eeUuCzXVasUVos

* Close the last open items on the live deletion test (ledger rows, email look, test account B deleted)

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018H7azoA9eeUuCzXVasUVos

---------

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/sprint/YOW-November-Launch-Sprint.xlsx
+++ b/docs/sprint/YOW-November-Launch-Sprint.xlsx
@@ -19,9 +19,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="ddd d mmm"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="13">
     <font>
@@ -2098,7 +2097,7 @@
       </c>
       <c r="L5" s="245" t="inlineStr">
         <is>
-          <t>Done 2026-10-01. Lifecycle built and tested: notices (Resend, ledger-first, max 20/run), grace, archive stamp (client reads cloud_archived_at), Free-account deletion (audit table, live re-check, media cleanup, max 10/run), all gated behind env settings + request flags and scheduled daily (09:15 UTC) inside the existing send-reengagement-emails function to stay within Vercel Hobby's 12 Functions. PRs 236-240; npm run qa 138 files / 1,349 tests, 0 lint errors. Migrations applied by owner. First production report: 160 accounts, 157 swept, 0 due. Notice wording owner-approved. Production edge/headers 22/22. Owner-reported live idle-logout and cross-tab auth checks passed. CARRIED to 3 Oct (O17): live end-to-end deletion test (no real email or deletion has run in production yet).</t>
+          <t>Done 2026-10-01. Lifecycle built and tested: notices (Resend, ledger-first, max 20/run), grace, archive stamp (client reads cloud_archived_at), Free-account deletion (audit table, live re-check, media cleanup, max 10/run), all gated behind env settings + request flags and scheduled daily (09:15 UTC) inside the existing send-reengagement-emails function to stay within Vercel Hobby's 12 Functions. PRs 236-240; npm run qa 138 files / 1,349 tests, 0 lint errors. Migrations applied by owner. First production report: 160 accounts, 157 swept, 0 due. Notice wording owner-approved. Production edge/headers 22/22. Owner-reported live idle-logout and cross-tab auth checks passed. The live end-to-end deletion test (O17) was run early and passed on 2 Oct.</t>
         </is>
       </c>
       <c r="M5" s="245" t="inlineStr">
@@ -2245,7 +2244,11 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="L7" s="245" t="inlineStr"/>
+      <c r="L7" s="245" t="inlineStr">
+        <is>
+          <t>O17 (Free-account deletion end-to-end) already done and passed on 2 Oct. See Owner Overflow O17 and docs/QA_PLAN.md. Remaining 3 Oct work is the rest of this day's assignment.</t>
+        </is>
+      </c>
       <c r="M7" s="245" t="inlineStr">
         <is>
           <t>2026-10-09</t>
@@ -11005,10 +11008,14 @@
       </c>
       <c r="H20" s="245" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="I20" s="245" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I20" s="245" t="inlineStr">
+        <is>
+          <t>Passed 2026-10-02 (run a day early). 8 notice emails arrived; cron run deleted test account A (audit row completed in 2 s, Storage folder gone); test account B signed in after the final notice and was not deleted; no real account touched. Found and fixed: Resend idempotency 409 (PR 243); emails restyled as branded HTML (PR 242). Owner confirmed B's ledger rows, the branded email look, and deleted test account B. No open items.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="C21" t="inlineStr">

</xml_diff>

<commit_message>
Update launch sprint spreadsheet for 2 Oct export work
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0158cVjiZnGqz1XKTCqNG8G1
</commit_message>
<xml_diff>
--- a/docs/sprint/YOW-November-Launch-Sprint.xlsx
+++ b/docs/sprint/YOW-November-Launch-Sprint.xlsx
@@ -1682,7 +1682,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1908,6 +1908,37 @@
       <c r="E10" s="245" t="inlineStr">
         <is>
           <t>O16</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="245" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B11" s="245" t="inlineStr">
+        <is>
+          <t>Check the new exports (about 15 min)</t>
+        </is>
+      </c>
+      <c r="C11" s="245" t="inlineStr">
+        <is>
+          <t>1. Open YOW (live site, after the update finishes deploying).
+2. Graphic Novel project: Project Settings &gt; Export &gt; PDF. Open it and confirm each comic page and its images are there.
+3. D&amp;D project: Export &gt; Word (ZIP). Open the Campaign Sessions file and confirm each encounter's text is under its session.
+4. Party &gt; click a character &gt; Download PDF (top right). Compare with the on-screen sheet.
+Tell Claude what looks wrong; do not fix anything yourself.</t>
+        </is>
+      </c>
+      <c r="D11" s="245" t="inlineStr">
+        <is>
+          <t>Live YOW site, Word or Google Docs</t>
+        </is>
+      </c>
+      <c r="E11" s="245" t="inlineStr">
+        <is>
+          <t>Plan from 1 Oct, 2 Oct</t>
         </is>
       </c>
     </row>
@@ -2166,10 +2197,14 @@
       </c>
       <c r="K6" s="245" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="L6" s="245" t="inlineStr"/>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="L6" s="245" t="inlineStr">
+        <is>
+          <t>In progress 2026-10-02. Fixed and merged (PR #247): Graphic Novel PDF now has the comic pages, panel text and page/panel images; D&amp;D Word export keeps each encounter's full text in the Campaign Sessions file; new party character sheet PDF (Download PDF button in Character Builder). Tests green (1,409). Still open: owner re-check of the Graphic Novel PDF, D&amp;D Word ZIP and character PDF; DOCX line-break check in real Word/Google Docs; AI-chat-to-Word check; World Bible/encyclopedia output for all six project types.</t>
+        </is>
+      </c>
       <c r="M6" s="245" t="inlineStr">
         <is>
           <t>2026-10-08</t>

</xml_diff>

<commit_message>
Update launch sprint spreadsheet for 2 Oct export work (#248)
Claude-Session: https://claude.ai/code/session_0158cVjiZnGqz1XKTCqNG8G1

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/sprint/YOW-November-Launch-Sprint.xlsx
+++ b/docs/sprint/YOW-November-Launch-Sprint.xlsx
@@ -1682,7 +1682,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1908,6 +1908,37 @@
       <c r="E10" s="245" t="inlineStr">
         <is>
           <t>O16</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="245" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B11" s="245" t="inlineStr">
+        <is>
+          <t>Check the new exports (about 15 min)</t>
+        </is>
+      </c>
+      <c r="C11" s="245" t="inlineStr">
+        <is>
+          <t>1. Open YOW (live site, after the update finishes deploying).
+2. Graphic Novel project: Project Settings &gt; Export &gt; PDF. Open it and confirm each comic page and its images are there.
+3. D&amp;D project: Export &gt; Word (ZIP). Open the Campaign Sessions file and confirm each encounter's text is under its session.
+4. Party &gt; click a character &gt; Download PDF (top right). Compare with the on-screen sheet.
+Tell Claude what looks wrong; do not fix anything yourself.</t>
+        </is>
+      </c>
+      <c r="D11" s="245" t="inlineStr">
+        <is>
+          <t>Live YOW site, Word or Google Docs</t>
+        </is>
+      </c>
+      <c r="E11" s="245" t="inlineStr">
+        <is>
+          <t>Plan from 1 Oct, 2 Oct</t>
         </is>
       </c>
     </row>
@@ -2166,10 +2197,14 @@
       </c>
       <c r="K6" s="245" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="L6" s="245" t="inlineStr"/>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="L6" s="245" t="inlineStr">
+        <is>
+          <t>In progress 2026-10-02. Fixed and merged (PR #247): Graphic Novel PDF now has the comic pages, panel text and page/panel images; D&amp;D Word export keeps each encounter's full text in the Campaign Sessions file; new party character sheet PDF (Download PDF button in Character Builder). Tests green (1,409). Still open: owner re-check of the Graphic Novel PDF, D&amp;D Word ZIP and character PDF; DOCX line-break check in real Word/Google Docs; AI-chat-to-Word check; World Bible/encyclopedia output for all six project types.</t>
+        </is>
+      </c>
       <c r="M6" s="245" t="inlineStr">
         <is>
           <t>2026-10-08</t>

</xml_diff>

<commit_message>
Mark 2 Oct export work Done after owner check
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0158cVjiZnGqz1XKTCqNG8G1
</commit_message>
<xml_diff>
--- a/docs/sprint/YOW-November-Launch-Sprint.xlsx
+++ b/docs/sprint/YOW-November-Launch-Sprint.xlsx
@@ -1919,7 +1919,7 @@
       </c>
       <c r="B11" s="245" t="inlineStr">
         <is>
-          <t>Check the new exports (about 15 min)</t>
+          <t>Check the new exports - DONE 2 Oct</t>
         </is>
       </c>
       <c r="C11" s="245" t="inlineStr">
@@ -1933,7 +1933,7 @@
       </c>
       <c r="D11" s="245" t="inlineStr">
         <is>
-          <t>Live YOW site, Word or Google Docs</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E11" s="245" t="inlineStr">
@@ -2197,12 +2197,12 @@
       </c>
       <c r="K6" s="245" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L6" s="245" t="inlineStr">
         <is>
-          <t>In progress 2026-10-02. Fixed and merged (PR #247): Graphic Novel PDF now has the comic pages, panel text and page/panel images; D&amp;D Word export keeps each encounter's full text in the Campaign Sessions file; new party character sheet PDF (Download PDF button in Character Builder). Tests green (1,409). Still open: owner re-check of the Graphic Novel PDF, D&amp;D Word ZIP and character PDF; DOCX line-break check in real Word/Google Docs; AI-chat-to-Word check; World Bible/encyclopedia output for all six project types.</t>
+          <t>Done 2026-10-02. Owner re-checked the new exports (Graphic Novel PDF, D&amp;D Word ZIP, character sheet PDF) on 2 Oct and confirmed they look good. Fixed and merged (PR #247): Graphic Novel PDF has comic pages, panel text and page/panel images; D&amp;D Word export keeps each encounter's full text in the Campaign Sessions file; party character sheet PDF added. Six-project-type export privacy matrix test merged (PR #249). D&amp;D Campaign renamed 5E Campaign in user-facing copy (PR #250).</t>
         </is>
       </c>
       <c r="M6" s="245" t="inlineStr">

</xml_diff>

<commit_message>
Mark 2 Oct export work Done after owner check (#251)
Claude-Session: https://claude.ai/code/session_0158cVjiZnGqz1XKTCqNG8G1

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/sprint/YOW-November-Launch-Sprint.xlsx
+++ b/docs/sprint/YOW-November-Launch-Sprint.xlsx
@@ -1919,7 +1919,7 @@
       </c>
       <c r="B11" s="245" t="inlineStr">
         <is>
-          <t>Check the new exports (about 15 min)</t>
+          <t>Check the new exports - DONE 2 Oct</t>
         </is>
       </c>
       <c r="C11" s="245" t="inlineStr">
@@ -1933,7 +1933,7 @@
       </c>
       <c r="D11" s="245" t="inlineStr">
         <is>
-          <t>Live YOW site, Word or Google Docs</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E11" s="245" t="inlineStr">
@@ -2197,12 +2197,12 @@
       </c>
       <c r="K6" s="245" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L6" s="245" t="inlineStr">
         <is>
-          <t>In progress 2026-10-02. Fixed and merged (PR #247): Graphic Novel PDF now has the comic pages, panel text and page/panel images; D&amp;D Word export keeps each encounter's full text in the Campaign Sessions file; new party character sheet PDF (Download PDF button in Character Builder). Tests green (1,409). Still open: owner re-check of the Graphic Novel PDF, D&amp;D Word ZIP and character PDF; DOCX line-break check in real Word/Google Docs; AI-chat-to-Word check; World Bible/encyclopedia output for all six project types.</t>
+          <t>Done 2026-10-02. Owner re-checked the new exports (Graphic Novel PDF, D&amp;D Word ZIP, character sheet PDF) on 2 Oct and confirmed they look good. Fixed and merged (PR #247): Graphic Novel PDF has comic pages, panel text and page/panel images; D&amp;D Word export keeps each encounter's full text in the Campaign Sessions file; party character sheet PDF added. Six-project-type export privacy matrix test merged (PR #249). D&amp;D Campaign renamed 5E Campaign in user-facing copy (PR #250).</t>
         </is>
       </c>
       <c r="M6" s="245" t="inlineStr">

</xml_diff>

<commit_message>
docs: owner sign-off 5 Oct (Data safety and Export ownership gates passed); record Stripe test results
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/sprint/YOW-November-Launch-Sprint.xlsx
+++ b/docs/sprint/YOW-November-Launch-Sprint.xlsx
@@ -1704,7 +1704,7 @@
     <row r="54" ht="229.85" customHeight="1" s="50">
       <c r="A54" s="62" t="inlineStr">
         <is>
-          <t>Updated 30 September: work starts 1 October. Use 'Do Now' first, then 'Plan from 1 Oct' as your daily sheet. Daily Guide rows after 6 Oct are marked Moved. Overflow checks are scheduled inside your daily caps; decisions D1-D8 accepted 30 Sep (AI providers: OpenRouter and OpenAI only). Updated 5 Oct: Daily Guide now ends at 5 Oct (6 Oct marked Moved); 'Plan from 1 Oct' is the only live schedule from 1 Oct and has been brought up to date through 5 Oct (3 and 4 Oct Done, 5 Oct awaiting your gate sign-off, 6-7 Oct partly pulled forward, pricing/Stripe test work recorded on 21-23 Oct).</t>
+          <t>Updated 30 September: work starts 1 October. Use 'Do Now' first, then 'Plan from 1 Oct' as your daily sheet. Daily Guide rows after 6 Oct are marked Moved. Overflow checks are scheduled inside your daily caps; decisions D1-D8 accepted 30 Sep (AI providers: OpenRouter and OpenAI only). Updated 5 Oct: Daily Guide now ends at 5 Oct (6 Oct marked Moved); 'Plan from 1 Oct' is the only live schedule from 1 Oct and has been brought up to date through 5 Oct (3 and 4 Oct Done, 5 Oct Done with both gates signed off, 6-7 Oct partly pulled forward, pricing/Stripe test work recorded on 21-23 Oct).</t>
         </is>
       </c>
     </row>
@@ -2469,12 +2469,12 @@
       </c>
       <c r="K9" s="65" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L9" s="65" t="inlineStr">
         <is>
-          <t>AI side done; owner sign-off outstanding. Data safety and Export ownership gate evidence summaries written 4 Oct (pulled forward at owner request; docs/QA_PLAN.md '2026-10-05 gate evidence summaries'); no known blocker, so both gates read 'Ready for owner sign-off' and move to Passed on your confirmation. O04 and O05 already Done (owner-reported 4 Oct). Security live checks done 5 Oct (original-plan work): headers, AI token rejection, durable AI logging and both form rate limits passed, no secrets in logs; email CORS fixes deployed with owner approval (reset v66, welcome v88, re-engagement v7), YOW origin allowed and attacker origin denied; security tests 74/74. Unplanned payment work done 5 Oct (scheduled 21-23 Oct, recorded there): simplified pricing to Free / Monthly GBP 10 / Lifetime, numbered Founder status (first 100 at GBP 50), private Stripe test checkout page, scheduled-cancellation display. To close this row: read the gate summaries and mark both gates Passed (or name the blocker).</t>
+          <t>Done 2026-10-05: owner signed off both gate summaries - Data safety gate and Export ownership gate PASSED. Data safety and Export ownership gate evidence summaries written 4 Oct (pulled forward at owner request; docs/QA_PLAN.md '2026-10-05 gate evidence summaries'); no known blocker, so both gates were signed off by the owner. O04 and O05 already Done (owner-reported 4 Oct). Security live checks done 5 Oct (original-plan work): headers, AI token rejection, durable AI logging and both form rate limits passed, no secrets in logs; email CORS fixes deployed with owner approval (reset v66, welcome v88, re-engagement v7), YOW origin allowed and attacker origin denied; security tests 74/74. Unplanned payment work done 5 Oct (scheduled 21-23 Oct, recorded there): simplified pricing to Free / Monthly GBP 10 / Lifetime, numbered Founder status (first 100 at GBP 50), private Stripe test checkout page, scheduled-cancellation display.</t>
         </is>
       </c>
       <c r="M9" s="65" t="inlineStr">
@@ -3526,7 +3526,7 @@
       </c>
       <c r="L26" s="65" t="inlineStr">
         <is>
-          <t>In progress 5 Oct 2026. Owner configured Stripe test products/prices, test environment variables and the deployed test webhook. The private direct-link billing page is live. Server-side Price validation and the transaction-locked Founder reservation/finalisation design are implemented and automated tests pass. Still open: live-mode final-position concurrency rehearsal, three-times event replay, refund/dispute handling, and final return-to-live review.</t>
+          <t>In progress 5 Oct 2026. Owner configured Stripe test products/prices, test environment variables and the deployed test webhook. The private direct-link billing page is live. Server-side Price validation and the transaction-locked Founder reservation/finalisation design are implemented and automated tests pass. Still open: live-mode final-position concurrency rehearsal, three-times event replay, refund/dispute handling, and final return-to-live review. Test-mode results are also logged in docs/PAYMENT_ROADMAP.md ('Test-mode QA results log').</t>
         </is>
       </c>
       <c r="M26" s="65" t="inlineStr">
@@ -3590,7 +3590,7 @@
       </c>
       <c r="L27" s="65" t="inlineStr">
         <is>
-          <t>Passed so far, owner-confirmed 5 Oct 2026: test-mode Monthly GBP 10 checkout and browser/Cloud entitlement; Founding Lifetime GBP 50 checkout; Standard Lifetime GBP 75 checkout; Monthly cancellation now reconciles directly with Stripe and shows the cancellation/end date; Monthly has no desktop entitlement. Supporting automated verification: 162 test files / 1,563 tests, zero lint errors, production build, 231-file load check and all 12 API imports. The remaining items in column E keep this row open.</t>
+          <t>Passed so far, owner-confirmed 5 Oct 2026: test-mode Monthly GBP 10 checkout and browser/Cloud entitlement; Founding Lifetime GBP 50 checkout; Standard Lifetime GBP 75 checkout; Monthly cancellation now reconciles directly with Stripe and shows the cancellation/end date; Monthly has no desktop entitlement. Supporting automated verification: 162 test files / 1,563 tests, zero lint errors, production build, 231-file load check and all 12 API imports. The remaining items in column E keep this row open. Logged in docs/PAYMENT_ROADMAP.md 'Test-mode QA results log'; open: live-mode reservation rehearsal (99/100/101), GBP 6 renewal, failure/expiry checks, 3x replay, refund/dispute, downgrade-fix live QA, return-to-live.</t>
         </is>
       </c>
       <c r="M27" s="65" t="inlineStr">
@@ -4902,7 +4902,7 @@
       </c>
       <c r="J18" s="87" t="inlineStr">
         <is>
-          <t>Done 2026-10-05. QA passed: 136/136 files, 1,244/1,244 tests, zero lint errors; security 74/74. Live checks passed for headers, AI token rejection, durable AI logging, and both form rate limits; no secrets appeared in logs. With owner approval, deployed email CORS fixes: reset v66, welcome v88, re-engagement v7. YOW origin allowed; attacker origin denied; auth/error behavior preserved; deployed source matched review. No email, AI completion, billing, customer-data, or public-content action. Broader gates remain separate. See also 'Plan from 1 Oct' 5 Oct row: gate summaries written, owner sign-off outstanding, and the 5 Oct pricing/Stripe test-checkout work.</t>
+          <t>Done 2026-10-05. QA passed: 136/136 files, 1,244/1,244 tests, zero lint errors; security 74/74. Live checks passed for headers, AI token rejection, durable AI logging, and both form rate limits; no secrets appeared in logs. With owner approval, deployed email CORS fixes: reset v66, welcome v88, re-engagement v7. YOW origin allowed; attacker origin denied; auth/error behavior preserved; deployed source matched review. No email, AI completion, billing, customer-data, or public-content action. Broader gates remain separate. See also 'Plan from 1 Oct' 5 Oct row: gate summaries written and signed off - Data safety and Export ownership gates Passed, and the 5 Oct pricing/Stripe test-checkout work.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sync sprint workbook statuses with roadmap (owner request)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JrE6DpPqhRXuHKSdowxCGC
</commit_message>
<xml_diff>
--- a/docs/sprint/YOW-November-Launch-Sprint.xlsx
+++ b/docs/sprint/YOW-November-Launch-Sprint.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet name="Start Here" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Open Items" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Plan from 1 Oct" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Daily Guide" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Calendar" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Glossary" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Roadmap Map" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Owner Overflow" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Decisions" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Items" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plan from 1 Oct" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily Guide" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calendar" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Glossary" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap Map" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Owner Overflow" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
 </workbook>
@@ -19,9 +19,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="ddd d mmm"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="13">
     <font>
@@ -1979,7 +1978,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Snapshot taken 12 Oct 2026. The roadmap is canonical; ask to regenerate this sheet after any change. Owner time per day is an estimate, push tasks to the next day when needed.</t>
+          <t>Statuses synced with docs/ROADMAP.md on 22 Oct 2026 (earlier dates in the text columns may be stale). The roadmap is canonical; ask to regenerate this sheet after any change.</t>
         </is>
       </c>
     </row>
@@ -2780,10 +2779,14 @@
       </c>
       <c r="J17" s="245" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="K17" s="245" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K17" s="245" t="inlineStr">
+        <is>
+          <t>Done 13 Oct - automated acceptance green; you reported the Novel and Comic journeys passed.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="246" t="n">
@@ -2831,10 +2834,14 @@
       </c>
       <c r="J18" s="245" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="K18" s="245" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K18" s="245" t="inlineStr">
+        <is>
+          <t>Done 14 Oct - Map Builder check run; grid fixed in code same day, re-check after deploy.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="246" t="n">
@@ -2882,10 +2889,14 @@
       </c>
       <c r="J19" s="245" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="K19" s="245" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K19" s="245" t="inlineStr">
+        <is>
+          <t>Done 16 Oct - automated checks green; you reported the live-account packet passed.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="246" t="n">
@@ -2933,10 +2944,14 @@
       </c>
       <c r="J20" s="245" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="K20" s="245" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K20" s="245" t="inlineStr">
+        <is>
+          <t>Done 18 Oct - Windows checklist passed on your real PC (installer hash comparison skipped).</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="246" t="n">
@@ -2984,10 +2999,14 @@
       </c>
       <c r="J21" s="245" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="K21" s="245" t="inlineStr"/>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="K21" s="245" t="inlineStr">
+        <is>
+          <t>Automated half done. Mobile/iPhone parked (decision D12). Still yours: desktop Safari/Firefox, keyboard-only and VoiceOver run (O10).</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="246" t="n">
@@ -3035,10 +3054,14 @@
       </c>
       <c r="J22" s="245" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="K22" s="245" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K22" s="245" t="inlineStr">
+        <is>
+          <t>Done - O07 (OpenRouter + OpenAI keys, two accounts, DM/GM framing) reported passed 19 Oct.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="246" t="n">
@@ -3086,10 +3109,14 @@
       </c>
       <c r="J23" s="245" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="K23" s="245" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K23" s="245" t="inlineStr">
+        <is>
+          <t>Done 19 Oct - Project-type gate closed; AI Import structure fixes deployed (PR #259).</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="246" t="n">
@@ -3137,10 +3164,14 @@
       </c>
       <c r="J24" s="245" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="K24" s="245" t="inlineStr"/>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="K24" s="245" t="inlineStr">
+        <is>
+          <t>AI-provider copy scrubbed and mobile promise fixed. Still to do (AI): Terms/Privacy fact check and COPY_CONFLICTS final pass.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="246" t="n">
@@ -3188,10 +3219,14 @@
       </c>
       <c r="J25" s="245" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="K25" s="245" t="inlineStr"/>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="K25" s="245" t="inlineStr">
+        <is>
+          <t>Checkout launch switch built (off), Stripe runbook written, tests green. You confirmed Stripe test config 22 Oct. Remaining: test-mode journey on 22 Oct.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="246" t="n">
@@ -9578,12 +9613,12 @@
       </c>
       <c r="H15" s="245" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="I15" s="245" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done 19 Oct - owner reported passed (no screenshots).</t>
         </is>
       </c>
     </row>
@@ -9619,12 +9654,12 @@
       </c>
       <c r="H16" s="245" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="I16" s="245" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>22 Oct: sitemap shows Success but last read 30 May (23 pages, bare domain). Needs www sitemap (15 pages) submitted.</t>
         </is>
       </c>
     </row>
@@ -9751,6 +9786,7 @@
         </is>
       </c>
     </row>
+    <row r="20"/>
     <row r="21">
       <c r="C21" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Record O11 Search Console sitemap done (22 Oct)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JrE6DpPqhRXuHKSdowxCGC
</commit_message>
<xml_diff>
--- a/docs/sprint/YOW-November-Launch-Sprint.xlsx
+++ b/docs/sprint/YOW-November-Launch-Sprint.xlsx
@@ -9654,12 +9654,12 @@
       </c>
       <c r="H16" s="245" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="I16" s="245" t="inlineStr">
         <is>
-          <t>22 Oct: sitemap shows Success but last read 30 May (23 pages, bare domain). Needs www sitemap (15 pages) submitted.</t>
+          <t>Done 22 Oct - www sitemap submitted in the Domain property; Success, 15 pages discovered (screenshot).</t>
         </is>
       </c>
     </row>

</xml_diff>